<commit_message>
qa: add 5 checks — contact name, cross-tab consistency, CLA01, X02, template placeholders
now 35 checks total (18 JB, 17 NA)

https://claude.ai/code/session_01USShV1LyhK3mB5ZoMsC9Cw
</commit_message>
<xml_diff>
--- a/LM Stats Briefing QA.xlsx
+++ b/LM Stats Briefing QA.xlsx
@@ -396,7 +396,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -657,6 +657,9 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="7" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3114,85 +3117,192 @@
       <c r="M39" s="63" t="n"/>
       <c r="N39" s="63" t="n"/>
     </row>
-    <row r="40" ht="125" customHeight="1">
+    <row r="40" ht="120" customHeight="1">
       <c r="A40" s="62" t="n"/>
-      <c r="B40" s="62" t="n"/>
-      <c r="C40" s="74" t="n"/>
-      <c r="D40" s="74" t="n"/>
-      <c r="E40" s="62" t="n"/>
-      <c r="F40" s="62" t="n"/>
-      <c r="G40" s="62" t="n"/>
-      <c r="H40" s="62" t="n"/>
-      <c r="I40" s="62" t="n"/>
-      <c r="J40" s="62" t="n"/>
-      <c r="K40" s="62" t="n"/>
-      <c r="L40" s="62" t="n"/>
-      <c r="M40" s="62" t="n"/>
-      <c r="N40" s="62" t="n"/>
-    </row>
-    <row r="41" ht="75" customHeight="1">
+      <c r="B40" s="72" t="inlineStr">
+        <is>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="C40" s="64" t="inlineStr">
+        <is>
+          <t>app.R + manual_word_output.R
+Contact name in Word header</t>
+        </is>
+      </c>
+      <c r="D40" s="65" t="inlineStr">
+        <is>
+          <t>Type a name in the contact input (e.g. 'Jane Smith and John Doe'). Download Word.
+• Open document — confirm header contains the entered name
+• Leave contact input blank — confirm header has no name (not 'qvzcontact' placeholder)
+• Check both Manual and Auto tabs pass contact_names correctly to generate_word_output / generate_manual_word_output</t>
+        </is>
+      </c>
+      <c r="E40" s="66" t="n"/>
+      <c r="F40" s="75" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G40" s="72" t="n"/>
+      <c r="H40" s="72" t="n"/>
+      <c r="I40" s="72" t="n"/>
+      <c r="J40" s="72" t="n"/>
+      <c r="K40" s="72" t="n"/>
+      <c r="L40" s="72" t="n"/>
+      <c r="M40" s="72" t="n"/>
+      <c r="N40" s="72" t="n"/>
+    </row>
+    <row r="41" ht="120" customHeight="1">
       <c r="A41" s="62" t="n"/>
-      <c r="B41" s="62" t="n"/>
-      <c r="C41" s="74" t="n"/>
-      <c r="D41" s="74" t="n"/>
-      <c r="E41" s="62" t="n"/>
-      <c r="F41" s="62" t="n"/>
-      <c r="G41" s="62" t="n"/>
-      <c r="H41" s="62" t="n"/>
-      <c r="I41" s="62" t="n"/>
-      <c r="J41" s="62" t="n"/>
-      <c r="K41" s="62" t="n"/>
-      <c r="L41" s="62" t="n"/>
-      <c r="M41" s="62" t="n"/>
-      <c r="N41" s="62" t="n"/>
-    </row>
-    <row r="42" ht="62.5" customHeight="1">
+      <c r="B41" s="72" t="inlineStr">
+        <is>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="C41" s="64" t="inlineStr">
+        <is>
+          <t>All files
+Manual vs Auto consistency</t>
+        </is>
+      </c>
+      <c r="D41" s="65" t="inlineStr">
+        <is>
+          <t>With DB connected and the same month's data available in both modes:
+• Run Preview Dashboard in both tabs — compare all metric values, confirm identical
+• Run Preview Top Ten in both tabs — compare all 10 lines, confirm identical
+• Run Preview Summary in both tabs — compare all lines, confirm identical
+• Download Word from both tabs — diff key figures, confirm they match
+Any discrepancy means the DB and Excel sources are out of sync, or the code paths diverge.</t>
+        </is>
+      </c>
+      <c r="E41" s="66" t="n"/>
+      <c r="F41" s="75" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G41" s="72" t="n"/>
+      <c r="H41" s="72" t="n"/>
+      <c r="I41" s="72" t="n"/>
+      <c r="J41" s="72" t="n"/>
+      <c r="K41" s="72" t="n"/>
+      <c r="L41" s="72" t="n"/>
+      <c r="M41" s="72" t="n"/>
+      <c r="N41" s="72" t="n"/>
+    </row>
+    <row r="42" ht="120" customHeight="1">
       <c r="A42" s="62" t="n"/>
-      <c r="B42" s="62" t="n"/>
-      <c r="C42" s="74" t="n"/>
-      <c r="D42" s="74" t="n"/>
-      <c r="E42" s="62" t="n"/>
-      <c r="F42" s="62" t="n"/>
-      <c r="G42" s="62" t="n"/>
-      <c r="H42" s="62" t="n"/>
-      <c r="I42" s="62" t="n"/>
-      <c r="J42" s="62" t="n"/>
-      <c r="K42" s="62" t="n"/>
-      <c r="L42" s="62" t="n"/>
-      <c r="M42" s="62" t="n"/>
-      <c r="N42" s="62" t="n"/>
-    </row>
-    <row r="43" ht="87.5" customHeight="1">
+      <c r="B42" s="72" t="inlineStr">
+        <is>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="C42" s="64" t="inlineStr">
+        <is>
+          <t>calculations_from_excel.R
+CLA01 — Claimant Count
+L467–510</t>
+        </is>
+      </c>
+      <c r="D42" s="65" t="inlineStr">
+        <is>
+          <t>Open CLA01, find latest period row.
+• Claimant count level → claimant_cur
+• Claimant rate → claimant_rt_cur
+• Month-on-month change → claimant_dm
+• Year-on-year change → claimant_dy
+Confirm these appear correctly in Preview Dashboard and in Top Ten / Summary lines that reference claimant count.</t>
+        </is>
+      </c>
+      <c r="E42" s="66" t="n"/>
+      <c r="F42" s="67" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G42" s="72" t="n"/>
+      <c r="H42" s="72" t="n"/>
+      <c r="I42" s="72" t="n"/>
+      <c r="J42" s="72" t="n"/>
+      <c r="K42" s="72" t="n"/>
+      <c r="L42" s="72" t="n"/>
+      <c r="M42" s="72" t="n"/>
+      <c r="N42" s="72" t="n"/>
+    </row>
+    <row r="43" ht="120" customHeight="1">
       <c r="A43" s="62" t="n"/>
-      <c r="B43" s="62" t="n"/>
-      <c r="C43" s="74" t="n"/>
-      <c r="D43" s="74" t="n"/>
-      <c r="E43" s="62" t="n"/>
-      <c r="F43" s="62" t="n"/>
-      <c r="G43" s="62" t="n"/>
-      <c r="H43" s="62" t="n"/>
-      <c r="I43" s="62" t="n"/>
-      <c r="J43" s="62" t="n"/>
-      <c r="K43" s="62" t="n"/>
-      <c r="L43" s="62" t="n"/>
-      <c r="M43" s="62" t="n"/>
-      <c r="N43" s="62" t="n"/>
-    </row>
-    <row r="44" ht="62.5" customHeight="1">
+      <c r="B43" s="72" t="inlineStr">
+        <is>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="C43" s="64" t="inlineStr">
+        <is>
+          <t>calculations_from_excel.R
+X02 — LFS flows
+Quarterly logic</t>
+        </is>
+      </c>
+      <c r="D43" s="65" t="inlineStr">
+        <is>
+          <t>Open X02 for the correct quarterly file (Feb/May/Aug/Nov cycle).
+• Confirm .build_ons_urls() picks the right quarterly month for the reference month
+• Spot-check flows figure against source file
+• If reference month is not a quarter month (e.g. March): confirm X02 URL points to most recent quarter (February)
+• Without X02 uploaded: confirm app handles gracefully</t>
+        </is>
+      </c>
+      <c r="E43" s="66" t="n"/>
+      <c r="F43" s="67" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G43" s="72" t="n"/>
+      <c r="H43" s="72" t="n"/>
+      <c r="I43" s="72" t="n"/>
+      <c r="J43" s="72" t="n"/>
+      <c r="K43" s="72" t="n"/>
+      <c r="L43" s="72" t="n"/>
+      <c r="M43" s="72" t="n"/>
+      <c r="N43" s="72" t="n"/>
+    </row>
+    <row r="44" ht="120" customHeight="1">
       <c r="A44" s="62" t="n"/>
-      <c r="B44" s="62" t="n"/>
-      <c r="C44" s="74" t="n"/>
-      <c r="D44" s="74" t="n"/>
-      <c r="E44" s="62" t="n"/>
-      <c r="F44" s="62" t="n"/>
-      <c r="G44" s="62" t="n"/>
-      <c r="H44" s="62" t="n"/>
-      <c r="I44" s="62" t="n"/>
-      <c r="J44" s="62" t="n"/>
-      <c r="K44" s="62" t="n"/>
-      <c r="L44" s="62" t="n"/>
-      <c r="M44" s="62" t="n"/>
-      <c r="N44" s="62" t="n"/>
+      <c r="B44" s="72" t="inlineStr">
+        <is>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="C44" s="64" t="inlineStr">
+        <is>
+          <t>utils/ManualDB.docx
+Template placeholders</t>
+        </is>
+      </c>
+      <c r="D44" s="65" t="inlineStr">
+        <is>
+          <t>Open ManualDB.docx in Word. Use Find &amp; Replace to search for 'qvz'.
+• List all qvz placeholders found — confirm each has a corresponding replace_all() call in manual_word_output.R
+• Check header: 'qvzcontact' present (not hardcoded names)
+• After generating a Word doc with all files uploaded: search output for 'qvz' — zero results means all placeholders were replaced</t>
+        </is>
+      </c>
+      <c r="E44" s="66" t="n"/>
+      <c r="F44" s="67" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G44" s="72" t="n"/>
+      <c r="H44" s="72" t="n"/>
+      <c r="I44" s="72" t="n"/>
+      <c r="J44" s="72" t="n"/>
+      <c r="K44" s="72" t="n"/>
+      <c r="L44" s="72" t="n"/>
+      <c r="M44" s="72" t="n"/>
+      <c r="N44" s="72" t="n"/>
     </row>
     <row r="45" ht="75" customHeight="1">
       <c r="A45" s="62" t="n"/>

</xml_diff>

<commit_message>
qa: remove CLA01 and X02 checks
now 33 checks (16 JB, 17 NA)

https://claude.ai/code/session_01USShV1LyhK3mB5ZoMsC9Cw
</commit_message>
<xml_diff>
--- a/LM Stats Briefing QA.xlsx
+++ b/LM Stats Briefing QA.xlsx
@@ -3200,19 +3200,16 @@
       </c>
       <c r="C42" s="64" t="inlineStr">
         <is>
-          <t>calculations_from_excel.R
-CLA01 — Claimant Count
-L467–510</t>
+          <t>utils/ManualDB.docx
+Template placeholders</t>
         </is>
       </c>
       <c r="D42" s="65" t="inlineStr">
         <is>
-          <t>Open CLA01, find latest period row.
-• Claimant count level → claimant_cur
-• Claimant rate → claimant_rt_cur
-• Month-on-month change → claimant_dm
-• Year-on-year change → claimant_dy
-Confirm these appear correctly in Preview Dashboard and in Top Ten / Summary lines that reference claimant count.</t>
+          <t>Open ManualDB.docx in Word. Use Find &amp; Replace to search for 'qvz'.
+• List all qvz placeholders found — confirm each has a corresponding replace_all() call in manual_word_output.R
+• Check header: 'qvzcontact' present (not hardcoded names)
+• After generating a Word doc with all files uploaded: search output for 'qvz' — zero results means all placeholders were replaced</t>
         </is>
       </c>
       <c r="E42" s="66" t="n"/>
@@ -3232,77 +3229,35 @@
     </row>
     <row r="43" ht="120" customHeight="1">
       <c r="A43" s="62" t="n"/>
-      <c r="B43" s="72" t="inlineStr">
-        <is>
-          <t>v0.1</t>
-        </is>
-      </c>
-      <c r="C43" s="64" t="inlineStr">
-        <is>
-          <t>calculations_from_excel.R
-X02 — LFS flows
-Quarterly logic</t>
-        </is>
-      </c>
-      <c r="D43" s="65" t="inlineStr">
-        <is>
-          <t>Open X02 for the correct quarterly file (Feb/May/Aug/Nov cycle).
-• Confirm .build_ons_urls() picks the right quarterly month for the reference month
-• Spot-check flows figure against source file
-• If reference month is not a quarter month (e.g. March): confirm X02 URL points to most recent quarter (February)
-• Without X02 uploaded: confirm app handles gracefully</t>
-        </is>
-      </c>
-      <c r="E43" s="66" t="n"/>
-      <c r="F43" s="67" t="inlineStr">
-        <is>
-          <t>JB</t>
-        </is>
-      </c>
-      <c r="G43" s="72" t="n"/>
-      <c r="H43" s="72" t="n"/>
-      <c r="I43" s="72" t="n"/>
-      <c r="J43" s="72" t="n"/>
-      <c r="K43" s="72" t="n"/>
-      <c r="L43" s="72" t="n"/>
-      <c r="M43" s="72" t="n"/>
-      <c r="N43" s="72" t="n"/>
+      <c r="B43" s="62" t="n"/>
+      <c r="C43" s="74" t="n"/>
+      <c r="D43" s="74" t="n"/>
+      <c r="E43" s="62" t="n"/>
+      <c r="F43" s="62" t="n"/>
+      <c r="G43" s="62" t="n"/>
+      <c r="H43" s="62" t="n"/>
+      <c r="I43" s="62" t="n"/>
+      <c r="J43" s="62" t="n"/>
+      <c r="K43" s="62" t="n"/>
+      <c r="L43" s="62" t="n"/>
+      <c r="M43" s="62" t="n"/>
+      <c r="N43" s="62" t="n"/>
     </row>
     <row r="44" ht="120" customHeight="1">
       <c r="A44" s="62" t="n"/>
-      <c r="B44" s="72" t="inlineStr">
-        <is>
-          <t>v0.1</t>
-        </is>
-      </c>
-      <c r="C44" s="64" t="inlineStr">
-        <is>
-          <t>utils/ManualDB.docx
-Template placeholders</t>
-        </is>
-      </c>
-      <c r="D44" s="65" t="inlineStr">
-        <is>
-          <t>Open ManualDB.docx in Word. Use Find &amp; Replace to search for 'qvz'.
-• List all qvz placeholders found — confirm each has a corresponding replace_all() call in manual_word_output.R
-• Check header: 'qvzcontact' present (not hardcoded names)
-• After generating a Word doc with all files uploaded: search output for 'qvz' — zero results means all placeholders were replaced</t>
-        </is>
-      </c>
-      <c r="E44" s="66" t="n"/>
-      <c r="F44" s="67" t="inlineStr">
-        <is>
-          <t>JB</t>
-        </is>
-      </c>
-      <c r="G44" s="72" t="n"/>
-      <c r="H44" s="72" t="n"/>
-      <c r="I44" s="72" t="n"/>
-      <c r="J44" s="72" t="n"/>
-      <c r="K44" s="72" t="n"/>
-      <c r="L44" s="72" t="n"/>
-      <c r="M44" s="72" t="n"/>
-      <c r="N44" s="72" t="n"/>
+      <c r="B44" s="62" t="n"/>
+      <c r="C44" s="74" t="n"/>
+      <c r="D44" s="74" t="n"/>
+      <c r="E44" s="62" t="n"/>
+      <c r="F44" s="62" t="n"/>
+      <c r="G44" s="62" t="n"/>
+      <c r="H44" s="62" t="n"/>
+      <c r="I44" s="62" t="n"/>
+      <c r="J44" s="62" t="n"/>
+      <c r="K44" s="62" t="n"/>
+      <c r="L44" s="62" t="n"/>
+      <c r="M44" s="62" t="n"/>
+      <c r="N44" s="62" t="n"/>
     </row>
     <row r="45" ht="75" customHeight="1">
       <c r="A45" s="62" t="n"/>
@@ -3352,38 +3307,8 @@
       <c r="M47" s="62" t="n"/>
       <c r="N47" s="62" t="n"/>
     </row>
-    <row r="48" ht="212.5" customHeight="1">
-      <c r="A48" s="62" t="n"/>
-      <c r="B48" s="62" t="n"/>
-      <c r="C48" s="74" t="n"/>
-      <c r="D48" s="74" t="n"/>
-      <c r="E48" s="62" t="n"/>
-      <c r="F48" s="62" t="n"/>
-      <c r="G48" s="62" t="n"/>
-      <c r="H48" s="62" t="n"/>
-      <c r="I48" s="62" t="n"/>
-      <c r="J48" s="62" t="n"/>
-      <c r="K48" s="62" t="n"/>
-      <c r="L48" s="62" t="n"/>
-      <c r="M48" s="62" t="n"/>
-      <c r="N48" s="62" t="n"/>
-    </row>
-    <row r="49" ht="75" customHeight="1">
-      <c r="A49" s="62" t="n"/>
-      <c r="B49" s="62" t="n"/>
-      <c r="C49" s="74" t="n"/>
-      <c r="D49" s="74" t="n"/>
-      <c r="E49" s="62" t="n"/>
-      <c r="F49" s="62" t="n"/>
-      <c r="G49" s="62" t="n"/>
-      <c r="H49" s="62" t="n"/>
-      <c r="I49" s="62" t="n"/>
-      <c r="J49" s="62" t="n"/>
-      <c r="K49" s="62" t="n"/>
-      <c r="L49" s="62" t="n"/>
-      <c r="M49" s="62" t="n"/>
-      <c r="N49" s="62" t="n"/>
-    </row>
+    <row r="48" ht="212.5" customHeight="1"/>
+    <row r="49" ht="75" customHeight="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="D7:K7"/>

</xml_diff>

<commit_message>
qa: add reference month input parsing check
tests various formats (March 2026, mar2026, gibberish, empty)
and confirms URLs update correctly. 34 checks (16 JB, 18 NA)

https://claude.ai/code/session_01USShV1LyhK3mB5ZoMsC9Cw
</commit_message>
<xml_diff>
--- a/LM Stats Briefing QA.xlsx
+++ b/LM Stats Briefing QA.xlsx
@@ -1783,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N49"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1796875" defaultRowHeight="12.5"/>
   <cols>
     <col width="2.81640625" customWidth="1" style="4" min="1" max="1"/>
@@ -3229,19 +3229,44 @@
     </row>
     <row r="43" ht="120" customHeight="1">
       <c r="A43" s="62" t="n"/>
-      <c r="B43" s="62" t="n"/>
-      <c r="C43" s="74" t="n"/>
-      <c r="D43" s="74" t="n"/>
-      <c r="E43" s="62" t="n"/>
-      <c r="F43" s="62" t="n"/>
-      <c r="G43" s="62" t="n"/>
-      <c r="H43" s="62" t="n"/>
-      <c r="I43" s="62" t="n"/>
-      <c r="J43" s="62" t="n"/>
-      <c r="K43" s="62" t="n"/>
-      <c r="L43" s="62" t="n"/>
-      <c r="M43" s="62" t="n"/>
-      <c r="N43" s="62" t="n"/>
+      <c r="B43" s="72" t="inlineStr">
+        <is>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="C43" s="64" t="inlineStr">
+        <is>
+          <t>app.R — Manual mode
+Reference month input parsing
+.parse_month_input() L1311–1327</t>
+        </is>
+      </c>
+      <c r="D43" s="65" t="inlineStr">
+        <is>
+          <t>Type each of these into the reference month field and confirm the download URLs and file tags update correctly:
+• 'March 2026' → recognised
+• 'march 2026' → recognised
+• 'Mar 2026' → recognised
+• 'mar2026' → recognised
+• 'gibberish' → no crash, URLs don't update
+• Empty string → no crash, Download All button still works (or is hidden)
+Confirm that after typing a valid month, the grey file tags link to correct ONS pages and Download All opens the right URLs.</t>
+        </is>
+      </c>
+      <c r="E43" s="66" t="n"/>
+      <c r="F43" s="75" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G43" s="72" t="n"/>
+      <c r="H43" s="72" t="n"/>
+      <c r="I43" s="72" t="n"/>
+      <c r="J43" s="72" t="n"/>
+      <c r="K43" s="72" t="n"/>
+      <c r="L43" s="72" t="n"/>
+      <c r="M43" s="72" t="n"/>
+      <c r="N43" s="72" t="n"/>
     </row>
     <row r="44" ht="120" customHeight="1">
       <c r="A44" s="62" t="n"/>

</xml_diff>

<commit_message>
Update QA spreadsheet for new OECD features
Updated checks 18, 35, 36, 42 to cover: G7 Average row, auto-generated
bullet points, ** stale period markers, UK ONS rate override, filtered
SDMX CSV parsing, NA fallback, and new template placeholders.

https://claude.ai/code/session_01USShV1LyhK3mB5ZoMsC9Cw
</commit_message>
<xml_diff>
--- a/LM Stats Briefing QA.xlsx
+++ b/LM Stats Briefing QA.xlsx
@@ -2285,15 +2285,17 @@
         <is>
           <t>manual_word_output.R
 OECD data parsing
-L20–90</t>
+L9–95 + word_helpers.R L279–370</t>
         </is>
       </c>
       <c r="D18" s="65" t="inlineStr">
         <is>
-          <t>Upload all 3 OECD files. Confirm .read_oecd_latest() returns a data frame with country, period, value columns.
+          <t>Upload all 3 OECD files (filtered CSV format). Confirm .read_oecd_latest() returns a data frame with country, period, value columns.
 • All 9 countries present: UK, US, France, Germany, Italy, Spain, Canada, Japan, Euro area
-• Period labels are human-readable (not raw SDMX codes)
+• Filtered SDMX CSV with paired code/label columns parsed correctly (code columns preferred)
 • Values formatted to 1dp
+• NA fallback: if latest quarter has NA, falls back to next available quarter
+• UK row uses ONS-derived rates (unemp_rt_cur, emp_rt_cur, inact_rt_cur) not OECD values
 Test with only 1 OECD file — confirm other columns show dash, no crash.</t>
         </is>
       </c>
@@ -2933,16 +2935,19 @@
         <is>
           <t>app.R — Manual mode
 Preview OECD rendering
-L2244–2310</t>
+L2290–2370</t>
         </is>
       </c>
       <c r="D35" s="65" t="inlineStr">
         <is>
-          <t>Upload all 3 OECD files. Preview OECD.
-• 9 country rows in order: UK, US, France, Germany, Italy, Spain, Canada, Japan, Euro Area
-• UK row has asterisk (*) on time period
+          <t>Upload all 3 OECD files + A01. Preview OECD.
+• 10 data rows in order: UK, US, France, Germany, Italy, Spain, Canada, Japan, G7 Average, Euro Area
+• UK row uses ONS rates (matches Dashboard values), time period has * suffix
+• G7 Average computed from 7 G7 countries (not Spain/Euro area)
+• Cells from older periods marked with ** and auto-generated ** footnote below table
+• 3 bullet points generated comparing UK to G7 (ranking, countries listed, ppts vs Euro Area/G7 avg)
 • Values formatted to 1dp with %
-• Footnote text present
+• Footnote text present including * and ** notes
 • Upload only unemployment file — other columns show dash not crash</t>
         </is>
       </c>
@@ -2981,7 +2986,10 @@
 • Filename: 'Labour Market Stats Briefing - March 2026.docx'
 • Opens cleanly (no Word repair prompt)
 • Search for 'qvz' — zero results (all placeholders replaced)
-• OECD table populated with 9 rows
+• OECD table: 10 data rows including G7 Average between Japan and Euro Area
+• UK row uses ONS rates, not OECD values
+• 3 bullet points below OECD footnotes with UK ranking text
+• ** footnote auto-generated if any cells use older period data
 • Contact name field blank or shows entered name
 • Spot-check 5 key figures against Preview Dashboard</t>
         </is>
@@ -3207,9 +3215,12 @@
       <c r="D42" s="65" t="inlineStr">
         <is>
           <t>Open ManualDB.docx in Word. Use Find &amp; Replace to search for 'qvz'.
-• List all qvz placeholders found — confirm each has a corresponding replace_all() call in manual_word_output.R
+• List all qvz placeholders found — confirm each has a corresponding replace_all() call
 • Check header: 'qvzcontact' present (not hardcoded names)
-• After generating a Word doc with all files uploaded: search output for 'qvz' — zero results means all placeholders were replaced</t>
+• OECD table: qvzoecdg7{tp,ur,er,ir} placeholders in G7 Average row
+• Bullet placeholders: qvzoecdbullet1, qvzoecdbullet2, qvzoecdbullet3
+• Stale note: qvzoecdstalenote placeholder for ** footnote
+• After generating a Word doc with all files uploaded: search output for 'qvz' — zero results</t>
         </is>
       </c>
       <c r="E42" s="66" t="n"/>

</xml_diff>

<commit_message>
Expand auto mode QA checks to cover OECD features thoroughly
Row 39 (auto full cycle): added OECD preview checks (G7 row, bullets,
** markers, UK from ONS), Word download OECD verification, Excel checks.
Row 41 (manual vs auto consistency): added OECD table, bullets, and **
marker comparison between tabs.

https://claude.ai/code/session_01USShV1LyhK3mB5ZoMsC9Cw
</commit_message>
<xml_diff>
--- a/LM Stats Briefing QA.xlsx
+++ b/LM Stats Briefing QA.xlsx
@@ -3104,9 +3104,21 @@
           <t>With DB connected:
 • Reference month auto-detected on launch
 • Period dropdowns populate with 2 options each, default to latest
-• Preview Dashboard, Top Ten, Summary — all render
-• Download Word — opens, figures populated, no placeholders
-• Download Excel — opens, sheets populated
+• Preview Dashboard — all metric rows populated, no dashes for available data
+• Preview Top Ten — 10 lines rendered, figures match Dashboard
+• Preview Summary — narrative renders, direction words match data
+• Preview OECD:
+  – 10 data rows: UK, US, France, Germany, Italy, Spain, Canada, Japan, G7 Average, Euro Area
+  – UK row uses ONS rates from DB (not OECD values), period has * suffix
+  – G7 Average row computed correctly
+  – Cells from older periods marked with **, auto-generated ** footnote
+  – 3 bullet points below: UK ranking in G7, ppts vs Euro Area/G7 averages
+• Download Word:
+  – Opens cleanly, no repair prompt
+  – Search 'qvz' — zero results
+  – OECD table has 10 rows including G7 Average
+  – 3 bullet points and ** footnote in Word match preview
+• Download Excel — opens, sheets populated, no repair prompt
 • DB unavailable: app launches without crash, informative message shown</t>
         </is>
       </c>
@@ -3177,11 +3189,15 @@
       <c r="D41" s="65" t="inlineStr">
         <is>
           <t>With DB connected and the same month's data available in both modes:
-• Run Preview Dashboard in both tabs — compare all metric values, confirm identical
-• Run Preview Top Ten in both tabs — compare all 10 lines, confirm identical
-• Run Preview Summary in both tabs — compare all lines, confirm identical
-• Download Word from both tabs — diff key figures, confirm they match
-Any discrepancy means the DB and Excel sources are out of sync, or the code paths diverge.</t>
+• Run Preview Dashboard in both tabs — compare all figures, they should match
+• Run Preview Top Ten in both tabs — all 10 lines identical
+• Run Preview Summary in both tabs — narrative text matches
+• Run Preview OECD in both tabs:
+  – Same 10 country rows with matching values
+  – UK row uses ONS rates in both (not OECD values)
+  – G7 Average and bullet points match
+  – ** markers and footnotes consistent
+• Download Word from both — diff the OECD table and bullet text</t>
         </is>
       </c>
       <c r="E41" s="66" t="n"/>

</xml_diff>

<commit_message>
Simplify auto mode QA — general checks without OECD specifics
https://claude.ai/code/session_01USShV1LyhK3mB5ZoMsC9Cw
</commit_message>
<xml_diff>
--- a/LM Stats Briefing QA.xlsx
+++ b/LM Stats Briefing QA.xlsx
@@ -3107,18 +3107,10 @@
 • Preview Dashboard — all metric rows populated, no dashes for available data
 • Preview Top Ten — 10 lines rendered, figures match Dashboard
 • Preview Summary — narrative renders, direction words match data
-• Preview OECD:
-  – 10 data rows: UK, US, France, Germany, Italy, Spain, Canada, Japan, G7 Average, Euro Area
-  – UK row uses ONS rates from DB (not OECD values), period has * suffix
-  – G7 Average row computed correctly
-  – Cells from older periods marked with **, auto-generated ** footnote
-  – 3 bullet points below: UK ranking in G7, ppts vs Euro Area/G7 averages
-• Download Word:
-  – Opens cleanly, no repair prompt
-  – Search 'qvz' — zero results
-  – OECD table has 10 rows including G7 Average
-  – 3 bullet points and ** footnote in Word match preview
+• Preview OECD — table renders with all countries, no crash
+• Download Word — opens cleanly, no repair prompt, search 'qvz' returns zero
 • Download Excel — opens, sheets populated, no repair prompt
+• Switch period buttons (vacancies, payroll) — previews update correctly
 • DB unavailable: app launches without crash, informative message shown</t>
         </is>
       </c>
@@ -3192,12 +3184,8 @@
 • Run Preview Dashboard in both tabs — compare all figures, they should match
 • Run Preview Top Ten in both tabs — all 10 lines identical
 • Run Preview Summary in both tabs — narrative text matches
-• Run Preview OECD in both tabs:
-  – Same 10 country rows with matching values
-  – UK row uses ONS rates in both (not OECD values)
-  – G7 Average and bullet points match
-  – ** markers and footnotes consistent
-• Download Word from both — diff the OECD table and bullet text</t>
+• Run Preview OECD in both tabs — table values match
+• Download Word from both — spot-check 5 key figures match</t>
         </is>
       </c>
       <c r="E41" s="66" t="n"/>

</xml_diff>

<commit_message>
Fix QA line number references to match current codebase
Line numbers drifted after OECD refactoring added ~70 lines to app.R.
Updated 14 rows: file detection, period buttons, download handlers,
preview renderers, auto mode, parse_month_input, and OECD sections.

https://claude.ai/code/session_01USShV1LyhK3mB5ZoMsC9Cw
</commit_message>
<xml_diff>
--- a/LM Stats Briefing QA.xlsx
+++ b/LM Stats Briefing QA.xlsx
@@ -2285,7 +2285,7 @@
         <is>
           <t>manual_word_output.R
 OECD data parsing
-L9–95 + word_helpers.R L279–370</t>
+L9–95 + word_helpers.R L279–396</t>
         </is>
       </c>
       <c r="D18" s="65" t="inlineStr">
@@ -2555,7 +2555,7 @@
         <is>
           <t>app.R — Manual mode
 File upload &amp; badge detection
-L750–816</t>
+L750–815</t>
         </is>
       </c>
       <c r="D25" s="65" t="inlineStr">
@@ -2593,7 +2593,7 @@
         <is>
           <t>app.R — Manual mode
 File detection fallback
-L670–742</t>
+L669–748</t>
         </is>
       </c>
       <c r="D26" s="65" t="inlineStr">
@@ -2740,7 +2740,7 @@
         <is>
           <t>app.R — Manual mode
 Vacancies period buttons
-L920–960</t>
+L920–967, L1024–1050</t>
         </is>
       </c>
       <c r="D30" s="65" t="inlineStr">
@@ -2780,7 +2780,7 @@
         <is>
           <t>app.R — Manual mode
 Payroll period buttons
-L960–1000</t>
+L969–1009, L1038–1050</t>
         </is>
       </c>
       <c r="D31" s="65" t="inlineStr">
@@ -2819,7 +2819,7 @@
         <is>
           <t>app.R — Manual mode
 Download All + file tags
-L856–918</t>
+L857–917</t>
         </is>
       </c>
       <c r="D32" s="65" t="inlineStr">
@@ -2857,7 +2857,7 @@
         <is>
           <t>app.R — Manual mode
 ONS download URLs
-.build_ons_urls() L817–852</t>
+.build_ons_urls() L818–851</t>
         </is>
       </c>
       <c r="D33" s="65" t="inlineStr">
@@ -2896,7 +2896,7 @@
         <is>
           <t>app.R — Manual mode
 Preview Dashboard rendering
-L2140–2201</t>
+L2211–2271</t>
         </is>
       </c>
       <c r="D34" s="65" t="inlineStr">
@@ -2935,7 +2935,7 @@
         <is>
           <t>app.R — Manual mode
 Preview OECD rendering
-L2290–2370</t>
+L2315–2395</t>
         </is>
       </c>
       <c r="D35" s="65" t="inlineStr">
@@ -2977,7 +2977,7 @@
         <is>
           <t>app.R — Manual mode
 Download Word
-L1972–2062</t>
+L2043–2132</t>
         </is>
       </c>
       <c r="D36" s="65" t="inlineStr">
@@ -3020,7 +3020,7 @@
         <is>
           <t>app.R — Manual mode
 Download Word — console
-L1972–2062</t>
+L2043–2132</t>
         </is>
       </c>
       <c r="D37" s="65" t="inlineStr">
@@ -3057,7 +3057,7 @@
         <is>
           <t>app.R — Manual mode
 Download Excel
-L2063–2139</t>
+L2134–2209</t>
         </is>
       </c>
       <c r="D38" s="65" t="inlineStr">
@@ -3096,7 +3096,7 @@
         <is>
           <t>app.R — Auto mode
 Full cycle with DB
-L1356–1669</t>
+L1357–1566</t>
         </is>
       </c>
       <c r="D39" s="65" t="inlineStr">
@@ -3253,7 +3253,7 @@
         <is>
           <t>app.R — Manual mode
 Reference month input parsing
-.parse_month_input() L1311–1327</t>
+.parse_month_input() L1319–1329</t>
         </is>
       </c>
       <c r="D43" s="65" t="inlineStr">

</xml_diff>

<commit_message>
qa: add granular function-level checks for JB
Append 138 new rows to AQA Log in LM Stats Briefing QA.xlsx — one QA item
per data-logic function across utils/ and sheets/. JB asked for finer
granularity so each function's logic gets an explicit check rather than
per-file block checks.

Each new row gives a one-line instruction (typically a direct R console
call with expected output), so JB can verify logic without going through
the app UI.

https://claude.ai/code/session_01FAPRDeoaRGPNKjn3Z3Mjdr
</commit_message>
<xml_diff>
--- a/LM Stats Briefing QA.xlsx
+++ b/LM Stats Briefing QA.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AQA Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AQA Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -677,7 +677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.81640625" customWidth="1" min="1" max="1"/>
@@ -714,7 +714,6 @@
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="5" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="13" customHeight="1">
       <c r="B4" s="6" t="inlineStr">
         <is>
@@ -799,7 +798,6 @@
       <c r="J7" s="9" t="n"/>
       <c r="K7" s="10" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9" ht="39" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
@@ -2177,69 +2175,4425 @@
       <c r="M43" s="20" t="n"/>
       <c r="N43" s="20" t="n"/>
     </row>
-    <row r="44" ht="120" customHeight="1">
+    <row r="44" ht="32" customHeight="1">
       <c r="A44" s="19" t="n"/>
-      <c r="B44" s="19" t="n"/>
-      <c r="C44" s="27" t="n"/>
-      <c r="D44" s="27" t="n"/>
-      <c r="E44" s="19" t="n"/>
-      <c r="F44" s="19" t="n"/>
-      <c r="G44" s="19" t="n"/>
-      <c r="H44" s="19" t="n"/>
-      <c r="I44" s="19" t="n"/>
-      <c r="J44" s="19" t="n"/>
-      <c r="K44" s="19" t="n"/>
-      <c r="L44" s="19" t="n"/>
-      <c r="M44" s="19" t="n"/>
-      <c r="N44" s="19" t="n"/>
-    </row>
-    <row r="45" ht="75" customHeight="1">
+      <c r="B44" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C44" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — auto_detect_manual_month
+L14</t>
+        </is>
+      </c>
+      <c r="D44" s="22" t="inlineStr">
+        <is>
+          <t>Run `auto_detect_manual_month()` with DB — returns anchor month e.g. "mar2026"; returns NULL without DB.</t>
+        </is>
+      </c>
+      <c r="E44" s="23" t="n"/>
+      <c r="F44" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G44" s="20" t="n"/>
+      <c r="H44" s="20" t="n"/>
+      <c r="I44" s="20" t="n"/>
+      <c r="J44" s="20" t="n"/>
+      <c r="K44" s="25" t="n"/>
+      <c r="L44" s="20" t="n"/>
+      <c r="M44" s="20" t="n"/>
+      <c r="N44" s="20" t="n"/>
+    </row>
+    <row r="45" ht="32" customHeight="1">
       <c r="A45" s="19" t="n"/>
-      <c r="B45" s="19" t="n"/>
-      <c r="C45" s="27" t="n"/>
-      <c r="D45" s="27" t="n"/>
-      <c r="E45" s="19" t="n"/>
-      <c r="F45" s="19" t="n"/>
-      <c r="G45" s="19" t="n"/>
-      <c r="H45" s="19" t="n"/>
-      <c r="I45" s="19" t="n"/>
-      <c r="J45" s="19" t="n"/>
-      <c r="K45" s="19" t="n"/>
-      <c r="L45" s="19" t="n"/>
-      <c r="M45" s="19" t="n"/>
-      <c r="N45" s="19" t="n"/>
-    </row>
-    <row r="46" ht="125" customHeight="1">
+      <c r="B45" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C45" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — parse_manual_month
+L45</t>
+        </is>
+      </c>
+      <c r="D45" s="22" t="inlineStr">
+        <is>
+          <t>Run `parse_manual_month("mar2026")` → 2026-03-01; "gibberish" → NULL; "" → NULL.</t>
+        </is>
+      </c>
+      <c r="E45" s="23" t="n"/>
+      <c r="F45" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G45" s="20" t="n"/>
+      <c r="H45" s="20" t="n"/>
+      <c r="I45" s="20" t="n"/>
+      <c r="J45" s="20" t="n"/>
+      <c r="K45" s="25" t="n"/>
+      <c r="L45" s="20" t="n"/>
+      <c r="M45" s="20" t="n"/>
+      <c r="N45" s="20" t="n"/>
+    </row>
+    <row r="46" ht="32" customHeight="1">
       <c r="A46" s="19" t="n"/>
-      <c r="B46" s="19" t="n"/>
-      <c r="C46" s="27" t="n"/>
-      <c r="D46" s="27" t="n"/>
-      <c r="E46" s="19" t="n"/>
-      <c r="F46" s="19" t="n"/>
-      <c r="G46" s="19" t="n"/>
-      <c r="H46" s="19" t="n"/>
-      <c r="I46" s="19" t="n"/>
-      <c r="J46" s="19" t="n"/>
-      <c r="K46" s="19" t="n"/>
-      <c r="L46" s="19" t="n"/>
-      <c r="M46" s="19" t="n"/>
-      <c r="N46" s="19" t="n"/>
-    </row>
-    <row r="47" ht="62.5" customHeight="1">
+      <c r="B46" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C46" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — make_lfs_label
+L57</t>
+        </is>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>Run `make_lfs_label(as.Date("2025-12-01"))` → "Oct-Dec 2025".</t>
+        </is>
+      </c>
+      <c r="E46" s="23" t="n"/>
+      <c r="F46" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G46" s="20" t="n"/>
+      <c r="H46" s="20" t="n"/>
+      <c r="I46" s="20" t="n"/>
+      <c r="J46" s="20" t="n"/>
+      <c r="K46" s="25" t="n"/>
+      <c r="L46" s="20" t="n"/>
+      <c r="M46" s="20" t="n"/>
+      <c r="N46" s="20" t="n"/>
+    </row>
+    <row r="47" ht="32" customHeight="1">
       <c r="A47" s="19" t="n"/>
-      <c r="B47" s="19" t="n"/>
-      <c r="C47" s="27" t="n"/>
-      <c r="D47" s="27" t="n"/>
-      <c r="E47" s="19" t="n"/>
-      <c r="F47" s="19" t="n"/>
-      <c r="G47" s="19" t="n"/>
-      <c r="H47" s="19" t="n"/>
-      <c r="I47" s="19" t="n"/>
-      <c r="J47" s="19" t="n"/>
-      <c r="K47" s="19" t="n"/>
-      <c r="L47" s="19" t="n"/>
-      <c r="M47" s="19" t="n"/>
-      <c r="N47" s="19" t="n"/>
+      <c r="B47" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C47" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — lfs_label_narrative
+L65</t>
+        </is>
+      </c>
+      <c r="D47" s="22" t="inlineStr">
+        <is>
+          <t>Run `lfs_label_narrative(as.Date("2025-12-01"))` → "October 2025 to December 2025".</t>
+        </is>
+      </c>
+      <c r="E47" s="23" t="n"/>
+      <c r="F47" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G47" s="20" t="n"/>
+      <c r="H47" s="20" t="n"/>
+      <c r="I47" s="20" t="n"/>
+      <c r="J47" s="20" t="n"/>
+      <c r="K47" s="25" t="n"/>
+      <c r="L47" s="20" t="n"/>
+      <c r="M47" s="20" t="n"/>
+      <c r="N47" s="20" t="n"/>
+    </row>
+    <row r="48" ht="32" customHeight="1">
+      <c r="B48" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C48" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — make_payroll_label
+L72</t>
+        </is>
+      </c>
+      <c r="D48" s="22" t="inlineStr">
+        <is>
+          <t>Run `make_payroll_label(as.Date("2025-03-01"))` → "March 2025".</t>
+        </is>
+      </c>
+      <c r="E48" s="23" t="n"/>
+      <c r="F48" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G48" s="20" t="n"/>
+      <c r="H48" s="20" t="n"/>
+      <c r="I48" s="20" t="n"/>
+      <c r="J48" s="20" t="n"/>
+      <c r="K48" s="25" t="n"/>
+      <c r="L48" s="20" t="n"/>
+      <c r="M48" s="20" t="n"/>
+      <c r="N48" s="20" t="n"/>
+    </row>
+    <row r="49" ht="32" customHeight="1">
+      <c r="B49" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C49" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — make_ymd_label
+L76</t>
+        </is>
+      </c>
+      <c r="D49" s="22" t="inlineStr">
+        <is>
+          <t>Run `make_ymd_label(as.Date("2025-03-01"))` → "2025-03-01".</t>
+        </is>
+      </c>
+      <c r="E49" s="23" t="n"/>
+      <c r="F49" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G49" s="20" t="n"/>
+      <c r="H49" s="20" t="n"/>
+      <c r="I49" s="20" t="n"/>
+      <c r="J49" s="20" t="n"/>
+      <c r="K49" s="25" t="n"/>
+      <c r="L49" s="20" t="n"/>
+      <c r="M49" s="20" t="n"/>
+      <c r="N49" s="20" t="n"/>
+    </row>
+    <row r="50" ht="32" customHeight="1">
+      <c r="B50" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — make_datetime_label
+L81</t>
+        </is>
+      </c>
+      <c r="D50" s="22" t="inlineStr">
+        <is>
+          <t>Run `make_datetime_label(as.Date("2025-03-01"))` → "2025-03-01 00:00:00".</t>
+        </is>
+      </c>
+      <c r="E50" s="23" t="n"/>
+      <c r="F50" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G50" s="20" t="n"/>
+      <c r="H50" s="20" t="n"/>
+      <c r="I50" s="20" t="n"/>
+      <c r="J50" s="20" t="n"/>
+      <c r="K50" s="25" t="n"/>
+      <c r="L50" s="20" t="n"/>
+      <c r="M50" s="20" t="n"/>
+      <c r="N50" s="20" t="n"/>
+    </row>
+    <row r="51" ht="32" customHeight="1">
+      <c r="B51" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C51" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — val_by_code
+L86</t>
+        </is>
+      </c>
+      <c r="D51" s="22" t="inlineStr">
+        <is>
+          <t>Returns NA_real_ when pg_data NULL/empty or code/period not matched; returns correct value on match.</t>
+        </is>
+      </c>
+      <c r="E51" s="23" t="n"/>
+      <c r="F51" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G51" s="20" t="n"/>
+      <c r="H51" s="20" t="n"/>
+      <c r="I51" s="20" t="n"/>
+      <c r="J51" s="20" t="n"/>
+      <c r="K51" s="25" t="n"/>
+      <c r="L51" s="20" t="n"/>
+      <c r="M51" s="20" t="n"/>
+      <c r="N51" s="20" t="n"/>
+    </row>
+    <row r="52" ht="32" customHeight="1">
+      <c r="B52" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C52" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — fmt_one_dec
+L95</t>
+        </is>
+      </c>
+      <c r="D52" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_one_dec(0.003)` → "0.003"; `fmt_one_dec(NA)` → "—".</t>
+        </is>
+      </c>
+      <c r="E52" s="23" t="n"/>
+      <c r="F52" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G52" s="20" t="n"/>
+      <c r="H52" s="20" t="n"/>
+      <c r="I52" s="20" t="n"/>
+      <c r="J52" s="20" t="n"/>
+      <c r="K52" s="25" t="n"/>
+      <c r="L52" s="20" t="n"/>
+      <c r="M52" s="20" t="n"/>
+      <c r="N52" s="20" t="n"/>
+    </row>
+    <row r="53" ht="32" customHeight="1">
+      <c r="B53" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C53" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — fmt_pct
+L106</t>
+        </is>
+      </c>
+      <c r="D53" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_pct(3.5)` → "3.5%"; `fmt_pct(NA)` → "—".</t>
+        </is>
+      </c>
+      <c r="E53" s="23" t="n"/>
+      <c r="F53" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G53" s="20" t="n"/>
+      <c r="H53" s="20" t="n"/>
+      <c r="I53" s="20" t="n"/>
+      <c r="J53" s="20" t="n"/>
+      <c r="K53" s="25" t="n"/>
+      <c r="L53" s="20" t="n"/>
+      <c r="M53" s="20" t="n"/>
+      <c r="N53" s="20" t="n"/>
+    </row>
+    <row r="54" ht="32" customHeight="1">
+      <c r="B54" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C54" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — fmt_pp
+L112</t>
+        </is>
+      </c>
+      <c r="D54" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_pp(0)` → "0.0 percentage points"; `fmt_pp(NA)` → "—".</t>
+        </is>
+      </c>
+      <c r="E54" s="23" t="n"/>
+      <c r="F54" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G54" s="20" t="n"/>
+      <c r="H54" s="20" t="n"/>
+      <c r="I54" s="20" t="n"/>
+      <c r="J54" s="20" t="n"/>
+      <c r="K54" s="25" t="n"/>
+      <c r="L54" s="20" t="n"/>
+      <c r="M54" s="20" t="n"/>
+      <c r="N54" s="20" t="n"/>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="B55" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C55" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — fmt_dir
+L119</t>
+        </is>
+      </c>
+      <c r="D55" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_dir(1)` → "up"; `fmt_dir(-1)` → "down"; `fmt_dir(0)` → "unchanged at"; `fmt_dir(NA)` → "".</t>
+        </is>
+      </c>
+      <c r="E55" s="23" t="n"/>
+      <c r="F55" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G55" s="20" t="n"/>
+      <c r="H55" s="20" t="n"/>
+      <c r="I55" s="20" t="n"/>
+      <c r="J55" s="20" t="n"/>
+      <c r="K55" s="25" t="n"/>
+      <c r="L55" s="20" t="n"/>
+      <c r="M55" s="20" t="n"/>
+      <c r="N55" s="20" t="n"/>
+    </row>
+    <row r="56" ht="32" customHeight="1">
+      <c r="B56" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C56" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — fmt_int
+L127</t>
+        </is>
+      </c>
+      <c r="D56" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_int(1234)` → "1,234"; `fmt_int(1e6)` → "1,000,000" (no scientific notation); `fmt_int(NA)` → "—".</t>
+        </is>
+      </c>
+      <c r="E56" s="23" t="n"/>
+      <c r="F56" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G56" s="20" t="n"/>
+      <c r="H56" s="20" t="n"/>
+      <c r="I56" s="20" t="n"/>
+      <c r="J56" s="20" t="n"/>
+      <c r="K56" s="25" t="n"/>
+      <c r="L56" s="20" t="n"/>
+      <c r="M56" s="20" t="n"/>
+      <c r="N56" s="20" t="n"/>
+    </row>
+    <row r="57" ht="32" customHeight="1">
+      <c r="B57" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C57" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — format_int
+L135</t>
+        </is>
+      </c>
+      <c r="D57" s="22" t="inlineStr">
+        <is>
+          <t>Run `format_int(1234)` → "+1,234"; `format_int(-500)` → "-500"; `format_int(0)` → "0".</t>
+        </is>
+      </c>
+      <c r="E57" s="23" t="n"/>
+      <c r="F57" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G57" s="20" t="n"/>
+      <c r="H57" s="20" t="n"/>
+      <c r="I57" s="20" t="n"/>
+      <c r="J57" s="20" t="n"/>
+      <c r="K57" s="25" t="n"/>
+      <c r="L57" s="20" t="n"/>
+      <c r="M57" s="20" t="n"/>
+      <c r="N57" s="20" t="n"/>
+    </row>
+    <row r="58" ht="32" customHeight="1">
+      <c r="B58" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C58" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — format_pp
+L143</t>
+        </is>
+      </c>
+      <c r="D58" s="22" t="inlineStr">
+        <is>
+          <t>Run `format_pp(0.03)` → "+0.03pp"; `format_pp(0)` → "0pp".</t>
+        </is>
+      </c>
+      <c r="E58" s="23" t="n"/>
+      <c r="F58" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G58" s="20" t="n"/>
+      <c r="H58" s="20" t="n"/>
+      <c r="I58" s="20" t="n"/>
+      <c r="J58" s="20" t="n"/>
+      <c r="K58" s="25" t="n"/>
+      <c r="L58" s="20" t="n"/>
+      <c r="M58" s="20" t="n"/>
+      <c r="N58" s="20" t="n"/>
+    </row>
+    <row r="59" ht="32" customHeight="1">
+      <c r="B59" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C59" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — format_pct1
+L155</t>
+        </is>
+      </c>
+      <c r="D59" s="22" t="inlineStr">
+        <is>
+          <t>Run `format_pct1(1.5)` → "+1.5%"; `format_pct1(0)` → "0%".</t>
+        </is>
+      </c>
+      <c r="E59" s="23" t="n"/>
+      <c r="F59" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G59" s="20" t="n"/>
+      <c r="H59" s="20" t="n"/>
+      <c r="I59" s="20" t="n"/>
+      <c r="J59" s="20" t="n"/>
+      <c r="K59" s="25" t="n"/>
+      <c r="L59" s="20" t="n"/>
+      <c r="M59" s="20" t="n"/>
+      <c r="N59" s="20" t="n"/>
+    </row>
+    <row r="60" ht="32" customHeight="1">
+      <c r="B60" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C60" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — format_gbp_signed0
+L167</t>
+        </is>
+      </c>
+      <c r="D60" s="22" t="inlineStr">
+        <is>
+          <t>Run `format_gbp_signed0(1234)` → "+£1,234"; `format_gbp_signed0(0)` → "£0".</t>
+        </is>
+      </c>
+      <c r="E60" s="23" t="n"/>
+      <c r="F60" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G60" s="20" t="n"/>
+      <c r="H60" s="20" t="n"/>
+      <c r="I60" s="20" t="n"/>
+      <c r="J60" s="20" t="n"/>
+      <c r="K60" s="25" t="n"/>
+      <c r="L60" s="20" t="n"/>
+      <c r="M60" s="20" t="n"/>
+      <c r="N60" s="20" t="n"/>
+    </row>
+    <row r="61" ht="32" customHeight="1">
+      <c r="B61" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C61" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — format_int_unsigned
+L177</t>
+        </is>
+      </c>
+      <c r="D61" s="22" t="inlineStr">
+        <is>
+          <t>Run `format_int_unsigned(-500)` → "500"; `format_int_unsigned(NA)` → NA.</t>
+        </is>
+      </c>
+      <c r="E61" s="23" t="n"/>
+      <c r="F61" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G61" s="20" t="n"/>
+      <c r="H61" s="20" t="n"/>
+      <c r="I61" s="20" t="n"/>
+      <c r="J61" s="20" t="n"/>
+      <c r="K61" s="25" t="n"/>
+      <c r="L61" s="20" t="n"/>
+      <c r="M61" s="20" t="n"/>
+      <c r="N61" s="20" t="n"/>
+    </row>
+    <row r="62" ht="32" customHeight="1">
+      <c r="B62" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C62" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — format_pct1_unsigned
+L184</t>
+        </is>
+      </c>
+      <c r="D62" s="22" t="inlineStr">
+        <is>
+          <t>Run `format_pct1_unsigned(-1.5)` → "1.5%"; `format_pct1_unsigned(0)` → "0.0%".</t>
+        </is>
+      </c>
+      <c r="E62" s="23" t="n"/>
+      <c r="F62" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G62" s="20" t="n"/>
+      <c r="H62" s="20" t="n"/>
+      <c r="I62" s="20" t="n"/>
+      <c r="J62" s="20" t="n"/>
+      <c r="K62" s="25" t="n"/>
+      <c r="L62" s="20" t="n"/>
+      <c r="M62" s="20" t="n"/>
+      <c r="N62" s="20" t="n"/>
+    </row>
+    <row r="63" ht="32" customHeight="1">
+      <c r="B63" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C63" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — safe_num
+L197</t>
+        </is>
+      </c>
+      <c r="D63" s="22" t="inlineStr">
+        <is>
+          <t>Run `safe_num("1.5")` → 1.5; `safe_num(NULL)` → NA_real_; `safe_num("abc")` → NA_real_.</t>
+        </is>
+      </c>
+      <c r="E63" s="23" t="n"/>
+      <c r="F63" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G63" s="20" t="n"/>
+      <c r="H63" s="20" t="n"/>
+      <c r="I63" s="20" t="n"/>
+      <c r="J63" s="20" t="n"/>
+      <c r="K63" s="25" t="n"/>
+      <c r="L63" s="20" t="n"/>
+      <c r="M63" s="20" t="n"/>
+      <c r="N63" s="20" t="n"/>
+    </row>
+    <row r="64" ht="32" customHeight="1">
+      <c r="B64" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C64" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — pct_from_delta
+L203</t>
+        </is>
+      </c>
+      <c r="D64" s="22" t="inlineStr">
+        <is>
+          <t>Run `pct_from_delta(110, 10)` → 10 (delta 10 on base 100); returns NA when base = 0.</t>
+        </is>
+      </c>
+      <c r="E64" s="23" t="n"/>
+      <c r="F64" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G64" s="20" t="n"/>
+      <c r="H64" s="20" t="n"/>
+      <c r="I64" s="20" t="n"/>
+      <c r="J64" s="20" t="n"/>
+      <c r="K64" s="25" t="n"/>
+      <c r="L64" s="20" t="n"/>
+      <c r="M64" s="20" t="n"/>
+      <c r="N64" s="20" t="n"/>
+    </row>
+    <row r="65" ht="32" customHeight="1">
+      <c r="B65" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C65" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — fmt_signed_int
+L210</t>
+        </is>
+      </c>
+      <c r="D65" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_signed_int(1234)` → "+1,234"; `fmt_signed_int(NA)` → "—".</t>
+        </is>
+      </c>
+      <c r="E65" s="23" t="n"/>
+      <c r="F65" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G65" s="20" t="n"/>
+      <c r="H65" s="20" t="n"/>
+      <c r="I65" s="20" t="n"/>
+      <c r="J65" s="20" t="n"/>
+      <c r="K65" s="25" t="n"/>
+      <c r="L65" s="20" t="n"/>
+      <c r="M65" s="20" t="n"/>
+      <c r="N65" s="20" t="n"/>
+    </row>
+    <row r="66" ht="32" customHeight="1">
+      <c r="B66" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C66" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — fmt_int_1k
+L216</t>
+        </is>
+      </c>
+      <c r="D66" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_int_1k(100000)` → "100,000" (no "1e+05"); `fmt_int_1k(NA)` → "—".</t>
+        </is>
+      </c>
+      <c r="E66" s="23" t="n"/>
+      <c r="F66" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G66" s="20" t="n"/>
+      <c r="H66" s="20" t="n"/>
+      <c r="I66" s="20" t="n"/>
+      <c r="J66" s="20" t="n"/>
+      <c r="K66" s="25" t="n"/>
+      <c r="L66" s="20" t="n"/>
+      <c r="M66" s="20" t="n"/>
+      <c r="N66" s="20" t="n"/>
+    </row>
+    <row r="67" ht="32" customHeight="1">
+      <c r="B67" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C67" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — fmt_signed_int_1k
+L221</t>
+        </is>
+      </c>
+      <c r="D67" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_signed_int_1k(1234)` → "+1,234"; `fmt_signed_int_1k(-1234)` → "-1,234".</t>
+        </is>
+      </c>
+      <c r="E67" s="23" t="n"/>
+      <c r="F67" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G67" s="20" t="n"/>
+      <c r="H67" s="20" t="n"/>
+      <c r="I67" s="20" t="n"/>
+      <c r="J67" s="20" t="n"/>
+      <c r="K67" s="25" t="n"/>
+      <c r="L67" s="20" t="n"/>
+      <c r="M67" s="20" t="n"/>
+      <c r="N67" s="20" t="n"/>
+    </row>
+    <row r="68" ht="32" customHeight="1">
+      <c r="B68" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C68" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — fmt_signed_pp
+L228</t>
+        </is>
+      </c>
+      <c r="D68" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_signed_pp(0.03)` → "+0.03 percentage points".</t>
+        </is>
+      </c>
+      <c r="E68" s="23" t="n"/>
+      <c r="F68" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G68" s="20" t="n"/>
+      <c r="H68" s="20" t="n"/>
+      <c r="I68" s="20" t="n"/>
+      <c r="J68" s="20" t="n"/>
+      <c r="K68" s="25" t="n"/>
+      <c r="L68" s="20" t="n"/>
+      <c r="M68" s="20" t="n"/>
+      <c r="N68" s="20" t="n"/>
+    </row>
+    <row r="69" ht="32" customHeight="1">
+      <c r="B69" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C69" s="21" t="inlineStr">
+        <is>
+          <t>helpers.R — fmt_pct_unsigned
+L241</t>
+        </is>
+      </c>
+      <c r="D69" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_pct_unsigned(-1.5)` → "1.5%".</t>
+        </is>
+      </c>
+      <c r="E69" s="23" t="n"/>
+      <c r="F69" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G69" s="20" t="n"/>
+      <c r="H69" s="20" t="n"/>
+      <c r="I69" s="20" t="n"/>
+      <c r="J69" s="20" t="n"/>
+      <c r="K69" s="25" t="n"/>
+      <c r="L69" s="20" t="n"/>
+      <c r="M69" s="20" t="n"/>
+      <c r="N69" s="20" t="n"/>
+    </row>
+    <row r="70" ht="32" customHeight="1">
+      <c r="B70" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C70" s="21" t="inlineStr">
+        <is>
+          <t>calculations_from_excel.R — .read_sheet
+L8</t>
+        </is>
+      </c>
+      <c r="D70" s="22" t="inlineStr">
+        <is>
+          <t>Call with bad path — returns empty data.frame, no crash, warning printed.</t>
+        </is>
+      </c>
+      <c r="E70" s="23" t="n"/>
+      <c r="F70" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G70" s="20" t="n"/>
+      <c r="H70" s="20" t="n"/>
+      <c r="I70" s="20" t="n"/>
+      <c r="J70" s="20" t="n"/>
+      <c r="K70" s="25" t="n"/>
+      <c r="L70" s="20" t="n"/>
+      <c r="M70" s="20" t="n"/>
+      <c r="N70" s="20" t="n"/>
+    </row>
+    <row r="71" ht="32" customHeight="1">
+      <c r="B71" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C71" s="21" t="inlineStr">
+        <is>
+          <t>calculations_from_excel.R — .safe_last
+L18</t>
+        </is>
+      </c>
+      <c r="D71" s="22" t="inlineStr">
+        <is>
+          <t>Run `.safe_last(c(1, NA, 3))` → 3; `.safe_last(c(NA, NA))` → NA_real_.</t>
+        </is>
+      </c>
+      <c r="E71" s="23" t="n"/>
+      <c r="F71" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G71" s="20" t="n"/>
+      <c r="H71" s="20" t="n"/>
+      <c r="I71" s="20" t="n"/>
+      <c r="J71" s="20" t="n"/>
+      <c r="K71" s="25" t="n"/>
+      <c r="L71" s="20" t="n"/>
+      <c r="M71" s="20" t="n"/>
+      <c r="N71" s="20" t="n"/>
+    </row>
+    <row r="72" ht="32" customHeight="1">
+      <c r="B72" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C72" s="21" t="inlineStr">
+        <is>
+          <t>calculations_from_excel.R — .find_col_by_code
+L25</t>
+        </is>
+      </c>
+      <c r="D72" s="22" t="inlineStr">
+        <is>
+          <t>Given a tbl where row 1 col 5 contains "KAC9", `.find_col_by_code(tbl, "KAC9")` → 5; unmatched code → fallback.</t>
+        </is>
+      </c>
+      <c r="E72" s="23" t="n"/>
+      <c r="F72" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G72" s="20" t="n"/>
+      <c r="H72" s="20" t="n"/>
+      <c r="I72" s="20" t="n"/>
+      <c r="J72" s="20" t="n"/>
+      <c r="K72" s="25" t="n"/>
+      <c r="L72" s="20" t="n"/>
+      <c r="M72" s="20" t="n"/>
+      <c r="N72" s="20" t="n"/>
+    </row>
+    <row r="73" ht="32" customHeight="1">
+      <c r="B73" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C73" s="21" t="inlineStr">
+        <is>
+          <t>calculations_from_excel.R — .detect_manual_month_from_a01
+L37</t>
+        </is>
+      </c>
+      <c r="D73" s="22" t="inlineStr">
+        <is>
+          <t>Given real A01 file path, returns "mmmYYYY" string matching LFS end + 2 months.</t>
+        </is>
+      </c>
+      <c r="E73" s="23" t="n"/>
+      <c r="F73" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G73" s="20" t="n"/>
+      <c r="H73" s="20" t="n"/>
+      <c r="I73" s="20" t="n"/>
+      <c r="J73" s="20" t="n"/>
+      <c r="K73" s="25" t="n"/>
+      <c r="L73" s="20" t="n"/>
+      <c r="M73" s="20" t="n"/>
+      <c r="N73" s="20" t="n"/>
+    </row>
+    <row r="74" ht="32" customHeight="1">
+      <c r="B74" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C74" s="21" t="inlineStr">
+        <is>
+          <t>calculations_from_excel.R — run_calculations_from_excel
+L59</t>
+        </is>
+      </c>
+      <c r="D74" s="22" t="inlineStr">
+        <is>
+          <t>Run with file_a01 = "A01.xls" — populates `emp16_cur`, `unemp16_cur`, `unemp_rt_cur`, `inact_cur`, `emp_rt_cur`, `inact_rt_cur` in globalenv.</t>
+        </is>
+      </c>
+      <c r="E74" s="23" t="n"/>
+      <c r="F74" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G74" s="20" t="n"/>
+      <c r="H74" s="20" t="n"/>
+      <c r="I74" s="20" t="n"/>
+      <c r="J74" s="20" t="n"/>
+      <c r="K74" s="25" t="n"/>
+      <c r="L74" s="20" t="n"/>
+      <c r="M74" s="20" t="n"/>
+      <c r="N74" s="20" t="n"/>
+    </row>
+    <row r="75" ht="32" customHeight="1">
+      <c r="B75" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C75" s="21" t="inlineStr">
+        <is>
+          <t>excel_helpers.R — .detect_dates
+L10</t>
+        </is>
+      </c>
+      <c r="D75" s="22" t="inlineStr">
+        <is>
+          <t>Parses Excel serial, datetime strings, and text dates correctly in the same vector.</t>
+        </is>
+      </c>
+      <c r="E75" s="23" t="n"/>
+      <c r="F75" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G75" s="20" t="n"/>
+      <c r="H75" s="20" t="n"/>
+      <c r="I75" s="20" t="n"/>
+      <c r="J75" s="20" t="n"/>
+      <c r="K75" s="25" t="n"/>
+      <c r="L75" s="20" t="n"/>
+      <c r="M75" s="20" t="n"/>
+      <c r="N75" s="20" t="n"/>
+    </row>
+    <row r="76" ht="32" customHeight="1">
+      <c r="B76" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C76" s="21" t="inlineStr">
+        <is>
+          <t>excel_helpers.R — .lfs_label
+L30</t>
+        </is>
+      </c>
+      <c r="D76" s="22" t="inlineStr">
+        <is>
+          <t>Run `.lfs_label(as.Date("2025-12-01"))` → "Oct-Dec 2025".</t>
+        </is>
+      </c>
+      <c r="E76" s="23" t="n"/>
+      <c r="F76" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G76" s="20" t="n"/>
+      <c r="H76" s="20" t="n"/>
+      <c r="I76" s="20" t="n"/>
+      <c r="J76" s="20" t="n"/>
+      <c r="K76" s="25" t="n"/>
+      <c r="L76" s="20" t="n"/>
+      <c r="M76" s="20" t="n"/>
+      <c r="N76" s="20" t="n"/>
+    </row>
+    <row r="77" ht="32" customHeight="1">
+      <c r="B77" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C77" s="21" t="inlineStr">
+        <is>
+          <t>excel_helpers.R — .find_row
+L36</t>
+        </is>
+      </c>
+      <c r="D77" s="22" t="inlineStr">
+        <is>
+          <t>Given tbl + label "Oct-Dec 2025", returns row index; returns NA when label absent.</t>
+        </is>
+      </c>
+      <c r="E77" s="23" t="n"/>
+      <c r="F77" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G77" s="20" t="n"/>
+      <c r="H77" s="20" t="n"/>
+      <c r="I77" s="20" t="n"/>
+      <c r="J77" s="20" t="n"/>
+      <c r="K77" s="25" t="n"/>
+      <c r="L77" s="20" t="n"/>
+      <c r="M77" s="20" t="n"/>
+      <c r="N77" s="20" t="n"/>
+    </row>
+    <row r="78" ht="32" customHeight="1">
+      <c r="B78" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C78" s="21" t="inlineStr">
+        <is>
+          <t>excel_helpers.R — .cell_num
+L46</t>
+        </is>
+      </c>
+      <c r="D78" s="22" t="inlineStr">
+        <is>
+          <t>`.cell_num(tbl, 5, 3)` returns numeric; non-numeric cell returns NA_real_.</t>
+        </is>
+      </c>
+      <c r="E78" s="23" t="n"/>
+      <c r="F78" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G78" s="20" t="n"/>
+      <c r="H78" s="20" t="n"/>
+      <c r="I78" s="20" t="n"/>
+      <c r="J78" s="20" t="n"/>
+      <c r="K78" s="25" t="n"/>
+      <c r="L78" s="20" t="n"/>
+      <c r="M78" s="20" t="n"/>
+      <c r="N78" s="20" t="n"/>
+    </row>
+    <row r="79" ht="32" customHeight="1">
+      <c r="B79" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C79" s="21" t="inlineStr">
+        <is>
+          <t>excel_helpers.R — .val_by_date
+L53</t>
+        </is>
+      </c>
+      <c r="D79" s="22" t="inlineStr">
+        <is>
+          <t>Returns matching value for target date; returns NA_real_ when date not found.</t>
+        </is>
+      </c>
+      <c r="E79" s="23" t="n"/>
+      <c r="F79" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G79" s="20" t="n"/>
+      <c r="H79" s="20" t="n"/>
+      <c r="I79" s="20" t="n"/>
+      <c r="J79" s="20" t="n"/>
+      <c r="K79" s="25" t="n"/>
+      <c r="L79" s="20" t="n"/>
+      <c r="M79" s="20" t="n"/>
+      <c r="N79" s="20" t="n"/>
+    </row>
+    <row r="80" ht="32" customHeight="1">
+      <c r="B80" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C80" s="21" t="inlineStr">
+        <is>
+          <t>excel_helpers.R — .avg_by_dates
+L60</t>
+        </is>
+      </c>
+      <c r="D80" s="22" t="inlineStr">
+        <is>
+          <t>`.avg_by_dates(df, c(d1, d2, d3))` returns mean across the 3 matching rows.</t>
+        </is>
+      </c>
+      <c r="E80" s="23" t="n"/>
+      <c r="F80" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G80" s="20" t="n"/>
+      <c r="H80" s="20" t="n"/>
+      <c r="I80" s="20" t="n"/>
+      <c r="J80" s="20" t="n"/>
+      <c r="K80" s="25" t="n"/>
+      <c r="L80" s="20" t="n"/>
+      <c r="M80" s="20" t="n"/>
+      <c r="N80" s="20" t="n"/>
+    </row>
+    <row r="81" ht="32" customHeight="1">
+      <c r="B81" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C81" s="21" t="inlineStr">
+        <is>
+          <t>manual_word_output.R — .read_oecd_latest
+L9</t>
+        </is>
+      </c>
+      <c r="D81" s="22" t="inlineStr">
+        <is>
+          <t>Accepts both SDMX CSV and wide Excel; returns df(country, period, value) with one latest non-NA row per country.</t>
+        </is>
+      </c>
+      <c r="E81" s="23" t="n"/>
+      <c r="F81" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G81" s="20" t="n"/>
+      <c r="H81" s="20" t="n"/>
+      <c r="I81" s="20" t="n"/>
+      <c r="J81" s="20" t="n"/>
+      <c r="K81" s="25" t="n"/>
+      <c r="L81" s="20" t="n"/>
+      <c r="M81" s="20" t="n"/>
+      <c r="N81" s="20" t="n"/>
+    </row>
+    <row r="82" ht="32" customHeight="1">
+      <c r="B82" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C82" s="21" t="inlineStr">
+        <is>
+          <t>manual_word_output.R — .parse_oecd_sdmx
+L66</t>
+        </is>
+      </c>
+      <c r="D82" s="22" t="inlineStr">
+        <is>
+          <t>Given SDMX CSV df with REF_AREA/TIME_PERIOD/OBS_VALUE columns, returns df(country, period, value) — one row per country.</t>
+        </is>
+      </c>
+      <c r="E82" s="23" t="n"/>
+      <c r="F82" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G82" s="20" t="n"/>
+      <c r="H82" s="20" t="n"/>
+      <c r="I82" s="20" t="n"/>
+      <c r="J82" s="20" t="n"/>
+      <c r="K82" s="25" t="n"/>
+      <c r="L82" s="20" t="n"/>
+      <c r="M82" s="20" t="n"/>
+      <c r="N82" s="20" t="n"/>
+    </row>
+    <row r="83" ht="32" customHeight="1">
+      <c r="B83" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C83" s="21" t="inlineStr">
+        <is>
+          <t>manual_word_output.R — generate_manual_word_output
+L97</t>
+        </is>
+      </c>
+      <c r="D83" s="22" t="inlineStr">
+        <is>
+          <t>Given all file paths + reference month, produces .docx with every `qvz` placeholder replaced (search output for "qvz" — zero hits).</t>
+        </is>
+      </c>
+      <c r="E83" s="23" t="n"/>
+      <c r="F83" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G83" s="20" t="n"/>
+      <c r="H83" s="20" t="n"/>
+      <c r="I83" s="20" t="n"/>
+      <c r="J83" s="20" t="n"/>
+      <c r="K83" s="25" t="n"/>
+      <c r="L83" s="20" t="n"/>
+      <c r="M83" s="20" t="n"/>
+      <c r="N83" s="20" t="n"/>
+    </row>
+    <row r="84" ht="32" customHeight="1">
+      <c r="B84" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C84" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — fmt_one_dec
+L13</t>
+        </is>
+      </c>
+      <c r="D84" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_one_dec(0.003)` → "0.003"; `fmt_one_dec(NA)` → "" (empty, not em-dash, for Word).</t>
+        </is>
+      </c>
+      <c r="E84" s="23" t="n"/>
+      <c r="F84" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G84" s="20" t="n"/>
+      <c r="H84" s="20" t="n"/>
+      <c r="I84" s="20" t="n"/>
+      <c r="J84" s="20" t="n"/>
+      <c r="K84" s="25" t="n"/>
+      <c r="L84" s="20" t="n"/>
+      <c r="M84" s="20" t="n"/>
+      <c r="N84" s="20" t="n"/>
+    </row>
+    <row r="85" ht="32" customHeight="1">
+      <c r="B85" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C85" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — .format_int
+L24</t>
+        </is>
+      </c>
+      <c r="D85" s="22" t="inlineStr">
+        <is>
+          <t>Delegates to format_int_unsigned when loaded; else uses scales::comma fallback.</t>
+        </is>
+      </c>
+      <c r="E85" s="23" t="n"/>
+      <c r="F85" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G85" s="20" t="n"/>
+      <c r="H85" s="20" t="n"/>
+      <c r="I85" s="20" t="n"/>
+      <c r="J85" s="20" t="n"/>
+      <c r="K85" s="25" t="n"/>
+      <c r="L85" s="20" t="n"/>
+      <c r="M85" s="20" t="n"/>
+      <c r="N85" s="20" t="n"/>
+    </row>
+    <row r="86" ht="32" customHeight="1">
+      <c r="B86" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C86" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — .format_pct
+L32</t>
+        </is>
+      </c>
+      <c r="D86" s="22" t="inlineStr">
+        <is>
+          <t>Run `.format_pct(1.5)` → "1.5%"; `.format_pct(NA)` → "" (empty).</t>
+        </is>
+      </c>
+      <c r="E86" s="23" t="n"/>
+      <c r="F86" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G86" s="20" t="n"/>
+      <c r="H86" s="20" t="n"/>
+      <c r="I86" s="20" t="n"/>
+      <c r="J86" s="20" t="n"/>
+      <c r="K86" s="25" t="n"/>
+      <c r="L86" s="20" t="n"/>
+      <c r="M86" s="20" t="n"/>
+      <c r="N86" s="20" t="n"/>
+    </row>
+    <row r="87" ht="32" customHeight="1">
+      <c r="B87" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C87" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — .format_pp
+L39</t>
+        </is>
+      </c>
+      <c r="D87" s="22" t="inlineStr">
+        <is>
+          <t>Run `.format_pp(0.5)` → "+0.5pp"; `.format_pp(0)` → "0.0pp".</t>
+        </is>
+      </c>
+      <c r="E87" s="23" t="n"/>
+      <c r="F87" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G87" s="20" t="n"/>
+      <c r="H87" s="20" t="n"/>
+      <c r="I87" s="20" t="n"/>
+      <c r="J87" s="20" t="n"/>
+      <c r="K87" s="25" t="n"/>
+      <c r="L87" s="20" t="n"/>
+      <c r="M87" s="20" t="n"/>
+      <c r="N87" s="20" t="n"/>
+    </row>
+    <row r="88" ht="32" customHeight="1">
+      <c r="B88" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C88" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — .format_gbp_signed0
+L47</t>
+        </is>
+      </c>
+      <c r="D88" s="22" t="inlineStr">
+        <is>
+          <t>Run `.format_gbp_signed0(1234)` → "+£1,234" (or fallback).</t>
+        </is>
+      </c>
+      <c r="E88" s="23" t="n"/>
+      <c r="F88" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G88" s="20" t="n"/>
+      <c r="H88" s="20" t="n"/>
+      <c r="I88" s="20" t="n"/>
+      <c r="J88" s="20" t="n"/>
+      <c r="K88" s="25" t="n"/>
+      <c r="L88" s="20" t="n"/>
+      <c r="M88" s="20" t="n"/>
+      <c r="N88" s="20" t="n"/>
+    </row>
+    <row r="89" ht="32" customHeight="1">
+      <c r="B89" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C89" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — fmt_int_signed
+L55</t>
+        </is>
+      </c>
+      <c r="D89" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_int_signed(-1234)` → "-1,234"; `fmt_int_signed(NA)` → "".</t>
+        </is>
+      </c>
+      <c r="E89" s="23" t="n"/>
+      <c r="F89" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G89" s="20" t="n"/>
+      <c r="H89" s="20" t="n"/>
+      <c r="I89" s="20" t="n"/>
+      <c r="J89" s="20" t="n"/>
+      <c r="K89" s="25" t="n"/>
+      <c r="L89" s="20" t="n"/>
+      <c r="M89" s="20" t="n"/>
+      <c r="N89" s="20" t="n"/>
+    </row>
+    <row r="90" ht="32" customHeight="1">
+      <c r="B90" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C90" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — fmt_count_000s_current
+L63</t>
+        </is>
+      </c>
+      <c r="D90" s="22" t="inlineStr">
+        <is>
+          <t>Divides input by 1000 then formats for narrative (e.g. 1500 → "1.5" or "2" per rounding).</t>
+        </is>
+      </c>
+      <c r="E90" s="23" t="n"/>
+      <c r="F90" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G90" s="20" t="n"/>
+      <c r="H90" s="20" t="n"/>
+      <c r="I90" s="20" t="n"/>
+      <c r="J90" s="20" t="n"/>
+      <c r="K90" s="25" t="n"/>
+      <c r="L90" s="20" t="n"/>
+      <c r="M90" s="20" t="n"/>
+      <c r="N90" s="20" t="n"/>
+    </row>
+    <row r="91" ht="32" customHeight="1">
+      <c r="B91" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C91" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — fmt_count_000s_change
+L64</t>
+        </is>
+      </c>
+      <c r="D91" s="22" t="inlineStr">
+        <is>
+          <t>Divides by 1000, applies sign, formats (e.g. -1500 → "-1.5" or signed thousands).</t>
+        </is>
+      </c>
+      <c r="E91" s="23" t="n"/>
+      <c r="F91" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G91" s="20" t="n"/>
+      <c r="H91" s="20" t="n"/>
+      <c r="I91" s="20" t="n"/>
+      <c r="J91" s="20" t="n"/>
+      <c r="K91" s="25" t="n"/>
+      <c r="L91" s="20" t="n"/>
+      <c r="M91" s="20" t="n"/>
+      <c r="N91" s="20" t="n"/>
+    </row>
+    <row r="92" ht="32" customHeight="1">
+      <c r="B92" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C92" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — fmt_exempt_current
+L67</t>
+        </is>
+      </c>
+      <c r="D92" s="22" t="inlineStr">
+        <is>
+          <t>Formats int without dividing (for already-in-thousands data).</t>
+        </is>
+      </c>
+      <c r="E92" s="23" t="n"/>
+      <c r="F92" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G92" s="20" t="n"/>
+      <c r="H92" s="20" t="n"/>
+      <c r="I92" s="20" t="n"/>
+      <c r="J92" s="20" t="n"/>
+      <c r="K92" s="25" t="n"/>
+      <c r="L92" s="20" t="n"/>
+      <c r="M92" s="20" t="n"/>
+      <c r="N92" s="20" t="n"/>
+    </row>
+    <row r="93" ht="32" customHeight="1">
+      <c r="B93" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C93" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — fmt_exempt_change
+L68</t>
+        </is>
+      </c>
+      <c r="D93" s="22" t="inlineStr">
+        <is>
+          <t>Signs int without dividing.</t>
+        </is>
+      </c>
+      <c r="E93" s="23" t="n"/>
+      <c r="F93" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G93" s="20" t="n"/>
+      <c r="H93" s="20" t="n"/>
+      <c r="I93" s="20" t="n"/>
+      <c r="J93" s="20" t="n"/>
+      <c r="K93" s="25" t="n"/>
+      <c r="L93" s="20" t="n"/>
+      <c r="M93" s="20" t="n"/>
+      <c r="N93" s="20" t="n"/>
+    </row>
+    <row r="94" ht="32" customHeight="1">
+      <c r="B94" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C94" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — manual_month_to_label
+L73</t>
+        </is>
+      </c>
+      <c r="D94" s="22" t="inlineStr">
+        <is>
+          <t>Run `manual_month_to_label("mar2026")` → "March 2026".</t>
+        </is>
+      </c>
+      <c r="E94" s="23" t="n"/>
+      <c r="F94" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G94" s="20" t="n"/>
+      <c r="H94" s="20" t="n"/>
+      <c r="I94" s="20" t="n"/>
+      <c r="J94" s="20" t="n"/>
+      <c r="K94" s="25" t="n"/>
+      <c r="L94" s="20" t="n"/>
+      <c r="M94" s="20" t="n"/>
+      <c r="N94" s="20" t="n"/>
+    </row>
+    <row r="95" ht="32" customHeight="1">
+      <c r="B95" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C95" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — replace_all
+L96</t>
+        </is>
+      </c>
+      <c r="D95" s="22" t="inlineStr">
+        <is>
+          <t>Replaces the placeholder string in body, headers, and footers of the docx; returns modified docx.</t>
+        </is>
+      </c>
+      <c r="E95" s="23" t="n"/>
+      <c r="F95" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G95" s="20" t="n"/>
+      <c r="H95" s="20" t="n"/>
+      <c r="I95" s="20" t="n"/>
+      <c r="J95" s="20" t="n"/>
+      <c r="K95" s="25" t="n"/>
+      <c r="L95" s="20" t="n"/>
+      <c r="M95" s="20" t="n"/>
+      <c r="N95" s="20" t="n"/>
+    </row>
+    <row r="96" ht="32" customHeight="1">
+      <c r="B96" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C96" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — fill_conditional
+L118</t>
+        </is>
+      </c>
+      <c r="D96" s="22" t="inlineStr">
+        <is>
+          <t>Picks the "+" variant when value ≥ 0, the "-" variant when value &lt; 0.</t>
+        </is>
+      </c>
+      <c r="E96" s="23" t="n"/>
+      <c r="F96" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G96" s="20" t="n"/>
+      <c r="H96" s="20" t="n"/>
+      <c r="I96" s="20" t="n"/>
+      <c r="J96" s="20" t="n"/>
+      <c r="K96" s="25" t="n"/>
+      <c r="L96" s="20" t="n"/>
+      <c r="M96" s="20" t="n"/>
+      <c r="N96" s="20" t="n"/>
+    </row>
+    <row r="97" ht="32" customHeight="1">
+      <c r="B97" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C97" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — .compute_g7_average
+L169</t>
+        </is>
+      </c>
+      <c r="D97" s="22" t="inlineStr">
+        <is>
+          <t>Given 3 OECD dfs, computes mean across UK/US/FR/DE/IT/CA/JP only — NOT Spain or Euro area.</t>
+        </is>
+      </c>
+      <c r="E97" s="23" t="n"/>
+      <c r="F97" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G97" s="20" t="n"/>
+      <c r="H97" s="20" t="n"/>
+      <c r="I97" s="20" t="n"/>
+      <c r="J97" s="20" t="n"/>
+      <c r="K97" s="25" t="n"/>
+      <c r="L97" s="20" t="n"/>
+      <c r="M97" s="20" t="n"/>
+      <c r="N97" s="20" t="n"/>
+    </row>
+    <row r="98" ht="32" customHeight="1">
+      <c r="B98" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C98" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — .generate_oecd_bullets
+L178</t>
+        </is>
+      </c>
+      <c r="D98" s="22" t="inlineStr">
+        <is>
+          <t>Returns 3-element list with UK ranking, country comparisons, and ppts deltas vs G7/EA.</t>
+        </is>
+      </c>
+      <c r="E98" s="23" t="n"/>
+      <c r="F98" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G98" s="20" t="n"/>
+      <c r="H98" s="20" t="n"/>
+      <c r="I98" s="20" t="n"/>
+      <c r="J98" s="20" t="n"/>
+      <c r="K98" s="25" t="n"/>
+      <c r="L98" s="20" t="n"/>
+      <c r="M98" s="20" t="n"/>
+      <c r="N98" s="20" t="n"/>
+    </row>
+    <row r="99" ht="32" customHeight="1">
+      <c r="B99" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C99" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — .manual_month_to_quarter
+L280</t>
+        </is>
+      </c>
+      <c r="D99" s="22" t="inlineStr">
+        <is>
+          <t>Run `.manual_month_to_quarter("mar2026")` → "Q1 2026".</t>
+        </is>
+      </c>
+      <c r="E99" s="23" t="n"/>
+      <c r="F99" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G99" s="20" t="n"/>
+      <c r="H99" s="20" t="n"/>
+      <c r="I99" s="20" t="n"/>
+      <c r="J99" s="20" t="n"/>
+      <c r="K99" s="25" t="n"/>
+      <c r="L99" s="20" t="n"/>
+      <c r="M99" s="20" t="n"/>
+      <c r="N99" s="20" t="n"/>
+    </row>
+    <row r="100" ht="32" customHeight="1">
+      <c r="B100" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C100" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — .get_uk_ons_overrides
+L292</t>
+        </is>
+      </c>
+      <c r="D100" s="22" t="inlineStr">
+        <is>
+          <t>Returns list with `unemp_rt_cur`, `emp_rt_cur`, `inact_rt_cur` sourced from globals.</t>
+        </is>
+      </c>
+      <c r="E100" s="23" t="n"/>
+      <c r="F100" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G100" s="20" t="n"/>
+      <c r="H100" s="20" t="n"/>
+      <c r="I100" s="20" t="n"/>
+      <c r="J100" s="20" t="n"/>
+      <c r="K100" s="25" t="n"/>
+      <c r="L100" s="20" t="n"/>
+      <c r="M100" s="20" t="n"/>
+      <c r="N100" s="20" t="n"/>
+    </row>
+    <row r="101" ht="32" customHeight="1">
+      <c r="B101" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C101" s="21" t="inlineStr">
+        <is>
+          <t>word_helpers.R — .fill_oecd_placeholders
+L303</t>
+        </is>
+      </c>
+      <c r="D101" s="22" t="inlineStr">
+        <is>
+          <t>Fills `qvzoecd{cc}{metric}`, G7 average placeholders, 3 bullet points, and stale-note footnote.</t>
+        </is>
+      </c>
+      <c r="E101" s="23" t="n"/>
+      <c r="F101" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G101" s="20" t="n"/>
+      <c r="H101" s="20" t="n"/>
+      <c r="I101" s="20" t="n"/>
+      <c r="J101" s="20" t="n"/>
+      <c r="K101" s="25" t="n"/>
+      <c r="L101" s="20" t="n"/>
+      <c r="M101" s="20" t="n"/>
+      <c r="N101" s="20" t="n"/>
+    </row>
+    <row r="102" ht="32" customHeight="1">
+      <c r="B102" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C102" s="21" t="inlineStr">
+        <is>
+          <t>word_output.R — .fetch_oecd_from_db
+L5</t>
+        </is>
+      </c>
+      <c r="D102" s="22" t="inlineStr">
+        <is>
+          <t>With DB connected, returns list(unemp, emp, inact) — each a df with country/period/value.</t>
+        </is>
+      </c>
+      <c r="E102" s="23" t="n"/>
+      <c r="F102" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G102" s="20" t="n"/>
+      <c r="H102" s="20" t="n"/>
+      <c r="I102" s="20" t="n"/>
+      <c r="J102" s="20" t="n"/>
+      <c r="K102" s="25" t="n"/>
+      <c r="L102" s="20" t="n"/>
+      <c r="M102" s="20" t="n"/>
+      <c r="N102" s="20" t="n"/>
+    </row>
+    <row r="103" ht="32" customHeight="1">
+      <c r="B103" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C103" s="21" t="inlineStr">
+        <is>
+          <t>word_output.R — generate_word_output
+L52</t>
+        </is>
+      </c>
+      <c r="D103" s="22" t="inlineStr">
+        <is>
+          <t>With DB + calculations loaded, produces .docx with all placeholders filled.</t>
+        </is>
+      </c>
+      <c r="E103" s="23" t="n"/>
+      <c r="F103" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G103" s="20" t="n"/>
+      <c r="H103" s="20" t="n"/>
+      <c r="I103" s="20" t="n"/>
+      <c r="J103" s="20" t="n"/>
+      <c r="K103" s="25" t="n"/>
+      <c r="L103" s="20" t="n"/>
+      <c r="M103" s="20" t="n"/>
+      <c r="N103" s="20" t="n"/>
+    </row>
+    <row r="104" ht="32" customHeight="1">
+      <c r="B104" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C104" s="21" t="inlineStr">
+        <is>
+          <t>calculations.R — .safe
+L21</t>
+        </is>
+      </c>
+      <c r="D104" s="22" t="inlineStr">
+        <is>
+          <t>Run `.safe(NULL, "a", "b")` → NA_real_; `.safe(list(a=list(b=5)), "a", "b")` → 5.</t>
+        </is>
+      </c>
+      <c r="E104" s="23" t="n"/>
+      <c r="F104" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G104" s="20" t="n"/>
+      <c r="H104" s="20" t="n"/>
+      <c r="I104" s="20" t="n"/>
+      <c r="J104" s="20" t="n"/>
+      <c r="K104" s="25" t="n"/>
+      <c r="L104" s="20" t="n"/>
+      <c r="M104" s="20" t="n"/>
+      <c r="N104" s="20" t="n"/>
+    </row>
+    <row r="105" ht="32" customHeight="1">
+      <c r="B105" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C105" s="21" t="inlineStr">
+        <is>
+          <t>calculations.R — .safe_chr
+L30</t>
+        </is>
+      </c>
+      <c r="D105" s="22" t="inlineStr">
+        <is>
+          <t>Returns NA_character_ on null/missing; correct string otherwise.</t>
+        </is>
+      </c>
+      <c r="E105" s="23" t="n"/>
+      <c r="F105" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G105" s="20" t="n"/>
+      <c r="H105" s="20" t="n"/>
+      <c r="I105" s="20" t="n"/>
+      <c r="J105" s="20" t="n"/>
+      <c r="K105" s="25" t="n"/>
+      <c r="L105" s="20" t="n"/>
+      <c r="M105" s="20" t="n"/>
+      <c r="N105" s="20" t="n"/>
+    </row>
+    <row r="106" ht="32" customHeight="1">
+      <c r="B106" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C106" s="21" t="inlineStr">
+        <is>
+          <t>calculations.R — .safe_date
+L39</t>
+        </is>
+      </c>
+      <c r="D106" s="22" t="inlineStr">
+        <is>
+          <t>Returns NA_date_ on null/missing; correct Date otherwise.</t>
+        </is>
+      </c>
+      <c r="E106" s="23" t="n"/>
+      <c r="F106" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G106" s="20" t="n"/>
+      <c r="H106" s="20" t="n"/>
+      <c r="I106" s="20" t="n"/>
+      <c r="J106" s="20" t="n"/>
+      <c r="K106" s="25" t="n"/>
+      <c r="L106" s="20" t="n"/>
+      <c r="M106" s="20" t="n"/>
+      <c r="N106" s="20" t="n"/>
+    </row>
+    <row r="107" ht="32" customHeight="1">
+      <c r="B107" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C107" s="21" t="inlineStr">
+        <is>
+          <t>sheets/lfs.R — fetch_lfs
+L14</t>
+        </is>
+      </c>
+      <c r="D107" s="22" t="inlineStr">
+        <is>
+          <t>With DB returns tibble(code, time_period, value); returns NULL if DB fails.</t>
+        </is>
+      </c>
+      <c r="E107" s="23" t="n"/>
+      <c r="F107" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G107" s="20" t="n"/>
+      <c r="H107" s="20" t="n"/>
+      <c r="I107" s="20" t="n"/>
+      <c r="J107" s="20" t="n"/>
+      <c r="K107" s="25" t="n"/>
+      <c r="L107" s="20" t="n"/>
+      <c r="M107" s="20" t="n"/>
+      <c r="N107" s="20" t="n"/>
+    </row>
+    <row r="108" ht="32" customHeight="1">
+      <c r="B108" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C108" s="21" t="inlineStr">
+        <is>
+          <t>sheets/lfs.R — compute_lfs_metric
+L28</t>
+        </is>
+      </c>
+      <c r="D108" s="22" t="inlineStr">
+        <is>
+          <t>Given code + df, returns list with cur/dq/dy/dc/de all numeric.</t>
+        </is>
+      </c>
+      <c r="E108" s="23" t="n"/>
+      <c r="F108" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G108" s="20" t="n"/>
+      <c r="H108" s="20" t="n"/>
+      <c r="I108" s="20" t="n"/>
+      <c r="J108" s="20" t="n"/>
+      <c r="K108" s="25" t="n"/>
+      <c r="L108" s="20" t="n"/>
+      <c r="M108" s="20" t="n"/>
+      <c r="N108" s="20" t="n"/>
+    </row>
+    <row r="109" ht="32" customHeight="1">
+      <c r="B109" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C109" s="21" t="inlineStr">
+        <is>
+          <t>sheets/lfs.R — calculate_lfs
+L50</t>
+        </is>
+      </c>
+      <c r="D109" s="22" t="inlineStr">
+        <is>
+          <t>Populates emp16, emp_rt, unemp16, unemp_rt, inact, inact_rt in target env.</t>
+        </is>
+      </c>
+      <c r="E109" s="23" t="n"/>
+      <c r="F109" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G109" s="20" t="n"/>
+      <c r="H109" s="20" t="n"/>
+      <c r="I109" s="20" t="n"/>
+      <c r="J109" s="20" t="n"/>
+      <c r="K109" s="25" t="n"/>
+      <c r="L109" s="20" t="n"/>
+      <c r="M109" s="20" t="n"/>
+      <c r="N109" s="20" t="n"/>
+    </row>
+    <row r="110" ht="32" customHeight="1">
+      <c r="B110" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C110" s="21" t="inlineStr">
+        <is>
+          <t>sheets/payroll.R — fetch_payroll
+L5</t>
+        </is>
+      </c>
+      <c r="D110" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble; NULL on DB failure.</t>
+        </is>
+      </c>
+      <c r="E110" s="23" t="n"/>
+      <c r="F110" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G110" s="20" t="n"/>
+      <c r="H110" s="20" t="n"/>
+      <c r="I110" s="20" t="n"/>
+      <c r="J110" s="20" t="n"/>
+      <c r="K110" s="25" t="n"/>
+      <c r="L110" s="20" t="n"/>
+      <c r="M110" s="20" t="n"/>
+      <c r="N110" s="20" t="n"/>
+    </row>
+    <row r="111" ht="32" customHeight="1">
+      <c r="B111" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C111" s="21" t="inlineStr">
+        <is>
+          <t>sheets/payroll.R — val_payroll
+L19</t>
+        </is>
+      </c>
+      <c r="D111" s="22" t="inlineStr">
+        <is>
+          <t>Returns numeric for month/unit match; NA_real_ on miss.</t>
+        </is>
+      </c>
+      <c r="E111" s="23" t="n"/>
+      <c r="F111" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G111" s="20" t="n"/>
+      <c r="H111" s="20" t="n"/>
+      <c r="I111" s="20" t="n"/>
+      <c r="J111" s="20" t="n"/>
+      <c r="K111" s="25" t="n"/>
+      <c r="L111" s="20" t="n"/>
+      <c r="M111" s="20" t="n"/>
+      <c r="N111" s="20" t="n"/>
+    </row>
+    <row r="112" ht="32" customHeight="1">
+      <c r="B112" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C112" s="21" t="inlineStr">
+        <is>
+          <t>sheets/payroll.R — get_payroll_avg
+L27</t>
+        </is>
+      </c>
+      <c r="D112" s="22" t="inlineStr">
+        <is>
+          <t>Returns mean of 3 consecutive months up to anchor.</t>
+        </is>
+      </c>
+      <c r="E112" s="23" t="n"/>
+      <c r="F112" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G112" s="20" t="n"/>
+      <c r="H112" s="20" t="n"/>
+      <c r="I112" s="20" t="n"/>
+      <c r="J112" s="20" t="n"/>
+      <c r="K112" s="25" t="n"/>
+      <c r="L112" s="20" t="n"/>
+      <c r="M112" s="20" t="n"/>
+      <c r="N112" s="20" t="n"/>
+    </row>
+    <row r="113" ht="32" customHeight="1">
+      <c r="B113" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C113" s="21" t="inlineStr">
+        <is>
+          <t>sheets/payroll.R — compute_payroll
+L33</t>
+        </is>
+      </c>
+      <c r="D113" s="22" t="inlineStr">
+        <is>
+          <t>Returns cur, flash_cur, _dm, _dy, _de for both anchor modes (aligned and latest).</t>
+        </is>
+      </c>
+      <c r="E113" s="23" t="n"/>
+      <c r="F113" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G113" s="20" t="n"/>
+      <c r="H113" s="20" t="n"/>
+      <c r="I113" s="20" t="n"/>
+      <c r="J113" s="20" t="n"/>
+      <c r="K113" s="25" t="n"/>
+      <c r="L113" s="20" t="n"/>
+      <c r="M113" s="20" t="n"/>
+      <c r="N113" s="20" t="n"/>
+    </row>
+    <row r="114" ht="32" customHeight="1">
+      <c r="B114" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C114" s="21" t="inlineStr">
+        <is>
+          <t>sheets/payroll.R — calculate_payroll
+L106</t>
+        </is>
+      </c>
+      <c r="D114" s="22" t="inlineStr">
+        <is>
+          <t>Populates `payroll_cur`, `payroll_flash_cur`, `payroll_flash_dy`, etc. in globals.</t>
+        </is>
+      </c>
+      <c r="E114" s="23" t="n"/>
+      <c r="F114" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G114" s="20" t="n"/>
+      <c r="H114" s="20" t="n"/>
+      <c r="I114" s="20" t="n"/>
+      <c r="J114" s="20" t="n"/>
+      <c r="K114" s="25" t="n"/>
+      <c r="L114" s="20" t="n"/>
+      <c r="M114" s="20" t="n"/>
+      <c r="N114" s="20" t="n"/>
+    </row>
+    <row r="115" ht="32" customHeight="1">
+      <c r="B115" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C115" s="21" t="inlineStr">
+        <is>
+          <t>sheets/vacancies.R — fetch_vacancies
+L8</t>
+        </is>
+      </c>
+      <c r="D115" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble with time_period/value.</t>
+        </is>
+      </c>
+      <c r="E115" s="23" t="n"/>
+      <c r="F115" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G115" s="20" t="n"/>
+      <c r="H115" s="20" t="n"/>
+      <c r="I115" s="20" t="n"/>
+      <c r="J115" s="20" t="n"/>
+      <c r="K115" s="25" t="n"/>
+      <c r="L115" s="20" t="n"/>
+      <c r="M115" s="20" t="n"/>
+      <c r="N115" s="20" t="n"/>
+    </row>
+    <row r="116" ht="32" customHeight="1">
+      <c r="B116" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C116" s="21" t="inlineStr">
+        <is>
+          <t>sheets/vacancies.R — parse_lfs_label_to_date
+L23</t>
+        </is>
+      </c>
+      <c r="D116" s="22" t="inlineStr">
+        <is>
+          <t>Run `parse_lfs_label_to_date("jul-sep 2025")` → 2025-09-01.</t>
+        </is>
+      </c>
+      <c r="E116" s="23" t="n"/>
+      <c r="F116" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G116" s="20" t="n"/>
+      <c r="H116" s="20" t="n"/>
+      <c r="I116" s="20" t="n"/>
+      <c r="J116" s="20" t="n"/>
+      <c r="K116" s="25" t="n"/>
+      <c r="L116" s="20" t="n"/>
+      <c r="M116" s="20" t="n"/>
+      <c r="N116" s="20" t="n"/>
+    </row>
+    <row r="117" ht="32" customHeight="1">
+      <c r="B117" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C117" s="21" t="inlineStr">
+        <is>
+          <t>sheets/vacancies.R — compute_vacancies
+L35</t>
+        </is>
+      </c>
+      <c r="D117" s="22" t="inlineStr">
+        <is>
+          <t>Returns cur/dq/dy/dc and `end` date for aligned or latest mode.</t>
+        </is>
+      </c>
+      <c r="E117" s="23" t="n"/>
+      <c r="F117" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G117" s="20" t="n"/>
+      <c r="H117" s="20" t="n"/>
+      <c r="I117" s="20" t="n"/>
+      <c r="J117" s="20" t="n"/>
+      <c r="K117" s="25" t="n"/>
+      <c r="L117" s="20" t="n"/>
+      <c r="M117" s="20" t="n"/>
+      <c r="N117" s="20" t="n"/>
+    </row>
+    <row r="118" ht="32" customHeight="1">
+      <c r="B118" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C118" s="21" t="inlineStr">
+        <is>
+          <t>sheets/vacancies.R — calculate_vacancies
+L89</t>
+        </is>
+      </c>
+      <c r="D118" s="22" t="inlineStr">
+        <is>
+          <t>Populates `vac`, `vac_cur`, `vac_dy`, `vac_dc` in globals.</t>
+        </is>
+      </c>
+      <c r="E118" s="23" t="n"/>
+      <c r="F118" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G118" s="20" t="n"/>
+      <c r="H118" s="20" t="n"/>
+      <c r="I118" s="20" t="n"/>
+      <c r="J118" s="20" t="n"/>
+      <c r="K118" s="25" t="n"/>
+      <c r="L118" s="20" t="n"/>
+      <c r="M118" s="20" t="n"/>
+      <c r="N118" s="20" t="n"/>
+    </row>
+    <row r="119" ht="32" customHeight="1">
+      <c r="B119" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C119" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_cpi.R — fetch_wages_cpi
+L17</t>
+        </is>
+      </c>
+      <c r="D119" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble from ons.labour_market__weekly_earnings_cpi.</t>
+        </is>
+      </c>
+      <c r="E119" s="23" t="n"/>
+      <c r="F119" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G119" s="20" t="n"/>
+      <c r="H119" s="20" t="n"/>
+      <c r="I119" s="20" t="n"/>
+      <c r="J119" s="20" t="n"/>
+      <c r="K119" s="25" t="n"/>
+      <c r="L119" s="20" t="n"/>
+      <c r="M119" s="20" t="n"/>
+      <c r="N119" s="20" t="n"/>
+    </row>
+    <row r="120" ht="32" customHeight="1">
+      <c r="B120" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C120" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_cpi.R — val_cpi_current
+L35</t>
+        </is>
+      </c>
+      <c r="D120" s="22" t="inlineStr">
+        <is>
+          <t>Returns YoY% 3mo avg for "total" or "regular" type.</t>
+        </is>
+      </c>
+      <c r="E120" s="23" t="n"/>
+      <c r="F120" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G120" s="20" t="n"/>
+      <c r="H120" s="20" t="n"/>
+      <c r="I120" s="20" t="n"/>
+      <c r="J120" s="20" t="n"/>
+      <c r="K120" s="25" t="n"/>
+      <c r="L120" s="20" t="n"/>
+      <c r="M120" s="20" t="n"/>
+      <c r="N120" s="20" t="n"/>
+    </row>
+    <row r="121" ht="32" customHeight="1">
+      <c r="B121" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C121" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_cpi.R — val_cpi_raw
+L49</t>
+        </is>
+      </c>
+      <c r="D121" s="22" t="inlineStr">
+        <is>
+          <t>Returns single-month real AWE £ value.</t>
+        </is>
+      </c>
+      <c r="E121" s="23" t="n"/>
+      <c r="F121" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G121" s="20" t="n"/>
+      <c r="H121" s="20" t="n"/>
+      <c r="I121" s="20" t="n"/>
+      <c r="J121" s="20" t="n"/>
+      <c r="K121" s="25" t="n"/>
+      <c r="L121" s="20" t="n"/>
+      <c r="M121" s="20" t="n"/>
+      <c r="N121" s="20" t="n"/>
+    </row>
+    <row r="122" ht="32" customHeight="1">
+      <c r="B122" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C122" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_cpi.R — get_cpi_raw_avg
+L62</t>
+        </is>
+      </c>
+      <c r="D122" s="22" t="inlineStr">
+        <is>
+          <t>Returns mean of 3 consecutive months of real AWE.</t>
+        </is>
+      </c>
+      <c r="E122" s="23" t="n"/>
+      <c r="F122" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G122" s="20" t="n"/>
+      <c r="H122" s="20" t="n"/>
+      <c r="I122" s="20" t="n"/>
+      <c r="J122" s="20" t="n"/>
+      <c r="K122" s="25" t="n"/>
+      <c r="L122" s="20" t="n"/>
+      <c r="M122" s="20" t="n"/>
+      <c r="N122" s="20" t="n"/>
+    </row>
+    <row r="123" ht="32" customHeight="1">
+      <c r="B123" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C123" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_cpi.R — compute_wages_cpi
+L68</t>
+        </is>
+      </c>
+      <c r="D123" s="22" t="inlineStr">
+        <is>
+          <t>Populates `latest_wages_cpi`, `latest_regular_cpi`, `wages_cpi_total_vs_dec2007`, `wages_cpi_total_vs_pandemic`.</t>
+        </is>
+      </c>
+      <c r="E123" s="23" t="n"/>
+      <c r="F123" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G123" s="20" t="n"/>
+      <c r="H123" s="20" t="n"/>
+      <c r="I123" s="20" t="n"/>
+      <c r="J123" s="20" t="n"/>
+      <c r="K123" s="25" t="n"/>
+      <c r="L123" s="20" t="n"/>
+      <c r="M123" s="20" t="n"/>
+      <c r="N123" s="20" t="n"/>
+    </row>
+    <row r="124" ht="32" customHeight="1">
+      <c r="B124" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C124" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_cpi.R — calculate_wages_cpi
+L126</t>
+        </is>
+      </c>
+      <c r="D124" s="22" t="inlineStr">
+        <is>
+          <t>Populates all CPI-adjusted wages globals.</t>
+        </is>
+      </c>
+      <c r="E124" s="23" t="n"/>
+      <c r="F124" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G124" s="20" t="n"/>
+      <c r="H124" s="20" t="n"/>
+      <c r="I124" s="20" t="n"/>
+      <c r="J124" s="20" t="n"/>
+      <c r="K124" s="25" t="n"/>
+      <c r="L124" s="20" t="n"/>
+      <c r="M124" s="20" t="n"/>
+      <c r="N124" s="20" t="n"/>
+    </row>
+    <row r="125" ht="32" customHeight="1">
+      <c r="B125" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C125" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_nominal.R — fetch_wages_total
+L14</t>
+        </is>
+      </c>
+      <c r="D125" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble from ons.labour_market__weekly_earnings_total.</t>
+        </is>
+      </c>
+      <c r="E125" s="23" t="n"/>
+      <c r="F125" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G125" s="20" t="n"/>
+      <c r="H125" s="20" t="n"/>
+      <c r="I125" s="20" t="n"/>
+      <c r="J125" s="20" t="n"/>
+      <c r="K125" s="25" t="n"/>
+      <c r="L125" s="20" t="n"/>
+      <c r="M125" s="20" t="n"/>
+      <c r="N125" s="20" t="n"/>
+    </row>
+    <row r="126" ht="32" customHeight="1">
+      <c r="B126" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C126" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_nominal.R — fetch_wages_regular
+L28</t>
+        </is>
+      </c>
+      <c r="D126" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble from ons.labour_market__weekly_earnings_regular.</t>
+        </is>
+      </c>
+      <c r="E126" s="23" t="n"/>
+      <c r="F126" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G126" s="20" t="n"/>
+      <c r="H126" s="20" t="n"/>
+      <c r="I126" s="20" t="n"/>
+      <c r="J126" s="20" t="n"/>
+      <c r="K126" s="25" t="n"/>
+      <c r="L126" s="20" t="n"/>
+      <c r="M126" s="20" t="n"/>
+      <c r="N126" s="20" t="n"/>
+    </row>
+    <row r="127" ht="32" customHeight="1">
+      <c r="B127" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C127" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_nominal.R — get_nom_val
+L42</t>
+        </is>
+      </c>
+      <c r="D127" s="22" t="inlineStr">
+        <is>
+          <t>Returns single-date value by code.</t>
+        </is>
+      </c>
+      <c r="E127" s="23" t="n"/>
+      <c r="F127" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G127" s="20" t="n"/>
+      <c r="H127" s="20" t="n"/>
+      <c r="I127" s="20" t="n"/>
+      <c r="J127" s="20" t="n"/>
+      <c r="K127" s="25" t="n"/>
+      <c r="L127" s="20" t="n"/>
+      <c r="M127" s="20" t="n"/>
+      <c r="N127" s="20" t="n"/>
+    </row>
+    <row r="128" ht="32" customHeight="1">
+      <c r="B128" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C128" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_nominal.R — get_nom_avg
+L46</t>
+        </is>
+      </c>
+      <c r="D128" s="22" t="inlineStr">
+        <is>
+          <t>Returns mean of 3 consecutive months.</t>
+        </is>
+      </c>
+      <c r="E128" s="23" t="n"/>
+      <c r="F128" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G128" s="20" t="n"/>
+      <c r="H128" s="20" t="n"/>
+      <c r="I128" s="20" t="n"/>
+      <c r="J128" s="20" t="n"/>
+      <c r="K128" s="25" t="n"/>
+      <c r="L128" s="20" t="n"/>
+      <c r="M128" s="20" t="n"/>
+      <c r="N128" s="20" t="n"/>
+    </row>
+    <row r="129" ht="32" customHeight="1">
+      <c r="B129" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C129" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_nominal.R — compute_wages_nominal
+L52</t>
+        </is>
+      </c>
+      <c r="D129" s="22" t="inlineStr">
+        <is>
+          <t>Populates `latest_wages`, `latest_regular_cash`, `wages_total_public`, `wages_total_private`, `wages_reg_public`, `wages_reg_private`.</t>
+        </is>
+      </c>
+      <c r="E129" s="23" t="n"/>
+      <c r="F129" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G129" s="20" t="n"/>
+      <c r="H129" s="20" t="n"/>
+      <c r="I129" s="20" t="n"/>
+      <c r="J129" s="20" t="n"/>
+      <c r="K129" s="25" t="n"/>
+      <c r="L129" s="20" t="n"/>
+      <c r="M129" s="20" t="n"/>
+      <c r="N129" s="20" t="n"/>
+    </row>
+    <row r="130" ht="32" customHeight="1">
+      <c r="B130" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C130" s="21" t="inlineStr">
+        <is>
+          <t>sheets/wages_nominal.R — calculate_wages_nominal
+L115</t>
+        </is>
+      </c>
+      <c r="D130" s="22" t="inlineStr">
+        <is>
+          <t>Populates all nominal wages globals.</t>
+        </is>
+      </c>
+      <c r="E130" s="23" t="n"/>
+      <c r="F130" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G130" s="20" t="n"/>
+      <c r="H130" s="20" t="n"/>
+      <c r="I130" s="20" t="n"/>
+      <c r="J130" s="20" t="n"/>
+      <c r="K130" s="25" t="n"/>
+      <c r="L130" s="20" t="n"/>
+      <c r="M130" s="20" t="n"/>
+      <c r="N130" s="20" t="n"/>
+    </row>
+    <row r="131" ht="32" customHeight="1">
+      <c r="B131" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C131" s="21" t="inlineStr">
+        <is>
+          <t>sheets/days_lost.R — fetch_days_lost
+L5</t>
+        </is>
+      </c>
+      <c r="D131" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble from ons.labour_market__disputes.</t>
+        </is>
+      </c>
+      <c r="E131" s="23" t="n"/>
+      <c r="F131" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G131" s="20" t="n"/>
+      <c r="H131" s="20" t="n"/>
+      <c r="I131" s="20" t="n"/>
+      <c r="J131" s="20" t="n"/>
+      <c r="K131" s="25" t="n"/>
+      <c r="L131" s="20" t="n"/>
+      <c r="M131" s="20" t="n"/>
+      <c r="N131" s="20" t="n"/>
+    </row>
+    <row r="132" ht="32" customHeight="1">
+      <c r="B132" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C132" s="21" t="inlineStr">
+        <is>
+          <t>sheets/days_lost.R — compute_days_lost
+L19</t>
+        </is>
+      </c>
+      <c r="D132" s="22" t="inlineStr">
+        <is>
+          <t>Returns single number for payroll-anchor month.</t>
+        </is>
+      </c>
+      <c r="E132" s="23" t="n"/>
+      <c r="F132" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G132" s="20" t="n"/>
+      <c r="H132" s="20" t="n"/>
+      <c r="I132" s="20" t="n"/>
+      <c r="J132" s="20" t="n"/>
+      <c r="K132" s="25" t="n"/>
+      <c r="L132" s="20" t="n"/>
+      <c r="M132" s="20" t="n"/>
+      <c r="N132" s="20" t="n"/>
+    </row>
+    <row r="133" ht="32" customHeight="1">
+      <c r="B133" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C133" s="21" t="inlineStr">
+        <is>
+          <t>sheets/days_lost.R — calculate_days_lost
+L32</t>
+        </is>
+      </c>
+      <c r="D133" s="22" t="inlineStr">
+        <is>
+          <t>Populates `days_lost_cur`, `days_lost_label` in globals.</t>
+        </is>
+      </c>
+      <c r="E133" s="23" t="n"/>
+      <c r="F133" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G133" s="20" t="n"/>
+      <c r="H133" s="20" t="n"/>
+      <c r="I133" s="20" t="n"/>
+      <c r="J133" s="20" t="n"/>
+      <c r="K133" s="25" t="n"/>
+      <c r="L133" s="20" t="n"/>
+      <c r="M133" s="20" t="n"/>
+      <c r="N133" s="20" t="n"/>
+    </row>
+    <row r="134" ht="32" customHeight="1">
+      <c r="B134" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C134" s="21" t="inlineStr">
+        <is>
+          <t>sheets/redundancy.R — fetch_redundancy
+L5</t>
+        </is>
+      </c>
+      <c r="D134" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble from ons.labour_market__redundancies.</t>
+        </is>
+      </c>
+      <c r="E134" s="23" t="n"/>
+      <c r="F134" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G134" s="20" t="n"/>
+      <c r="H134" s="20" t="n"/>
+      <c r="I134" s="20" t="n"/>
+      <c r="J134" s="20" t="n"/>
+      <c r="K134" s="25" t="n"/>
+      <c r="L134" s="20" t="n"/>
+      <c r="M134" s="20" t="n"/>
+      <c r="N134" s="20" t="n"/>
+    </row>
+    <row r="135" ht="32" customHeight="1">
+      <c r="B135" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C135" s="21" t="inlineStr">
+        <is>
+          <t>sheets/redundancy.R — compute_redundancy
+L19</t>
+        </is>
+      </c>
+      <c r="D135" s="22" t="inlineStr">
+        <is>
+          <t>Returns cur/dq/dy/dc/de using COVID + election baselines.</t>
+        </is>
+      </c>
+      <c r="E135" s="23" t="n"/>
+      <c r="F135" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G135" s="20" t="n"/>
+      <c r="H135" s="20" t="n"/>
+      <c r="I135" s="20" t="n"/>
+      <c r="J135" s="20" t="n"/>
+      <c r="K135" s="25" t="n"/>
+      <c r="L135" s="20" t="n"/>
+      <c r="M135" s="20" t="n"/>
+      <c r="N135" s="20" t="n"/>
+    </row>
+    <row r="136" ht="32" customHeight="1">
+      <c r="B136" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C136" s="21" t="inlineStr">
+        <is>
+          <t>sheets/redundancy.R — calculate_redundancy
+L45</t>
+        </is>
+      </c>
+      <c r="D136" s="22" t="inlineStr">
+        <is>
+          <t>Populates `redund_cur`, `redund_level_cur`, `redund_dq`, `redund_dy` in globals.</t>
+        </is>
+      </c>
+      <c r="E136" s="23" t="n"/>
+      <c r="F136" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G136" s="20" t="n"/>
+      <c r="H136" s="20" t="n"/>
+      <c r="I136" s="20" t="n"/>
+      <c r="J136" s="20" t="n"/>
+      <c r="K136" s="25" t="n"/>
+      <c r="L136" s="20" t="n"/>
+      <c r="M136" s="20" t="n"/>
+      <c r="N136" s="20" t="n"/>
+    </row>
+    <row r="137" ht="32" customHeight="1">
+      <c r="B137" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C137" s="21" t="inlineStr">
+        <is>
+          <t>sheets/hr1.R — fetch_hr1
+L5</t>
+        </is>
+      </c>
+      <c r="D137" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble from ons.labour_market__redundancies_region.</t>
+        </is>
+      </c>
+      <c r="E137" s="23" t="n"/>
+      <c r="F137" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G137" s="20" t="n"/>
+      <c r="H137" s="20" t="n"/>
+      <c r="I137" s="20" t="n"/>
+      <c r="J137" s="20" t="n"/>
+      <c r="K137" s="25" t="n"/>
+      <c r="L137" s="20" t="n"/>
+      <c r="M137" s="20" t="n"/>
+      <c r="N137" s="20" t="n"/>
+    </row>
+    <row r="138" ht="32" customHeight="1">
+      <c r="B138" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C138" s="21" t="inlineStr">
+        <is>
+          <t>sheets/hr1.R — val_hr1
+L19</t>
+        </is>
+      </c>
+      <c r="D138" s="22" t="inlineStr">
+        <is>
+          <t>Returns numeric for period/region combo.</t>
+        </is>
+      </c>
+      <c r="E138" s="23" t="n"/>
+      <c r="F138" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G138" s="20" t="n"/>
+      <c r="H138" s="20" t="n"/>
+      <c r="I138" s="20" t="n"/>
+      <c r="J138" s="20" t="n"/>
+      <c r="K138" s="25" t="n"/>
+      <c r="L138" s="20" t="n"/>
+      <c r="M138" s="20" t="n"/>
+      <c r="N138" s="20" t="n"/>
+    </row>
+    <row r="139" ht="32" customHeight="1">
+      <c r="B139" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C139" s="21" t="inlineStr">
+        <is>
+          <t>sheets/hr1.R — compute_hr1
+L26</t>
+        </is>
+      </c>
+      <c r="D139" s="22" t="inlineStr">
+        <is>
+          <t>Returns cur/dm/dy/dc/de.</t>
+        </is>
+      </c>
+      <c r="E139" s="23" t="n"/>
+      <c r="F139" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G139" s="20" t="n"/>
+      <c r="H139" s="20" t="n"/>
+      <c r="I139" s="20" t="n"/>
+      <c r="J139" s="20" t="n"/>
+      <c r="K139" s="25" t="n"/>
+      <c r="L139" s="20" t="n"/>
+      <c r="M139" s="20" t="n"/>
+      <c r="N139" s="20" t="n"/>
+    </row>
+    <row r="140" ht="32" customHeight="1">
+      <c r="B140" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C140" s="21" t="inlineStr">
+        <is>
+          <t>sheets/hr1.R — calculate_hr1
+L59</t>
+        </is>
+      </c>
+      <c r="D140" s="22" t="inlineStr">
+        <is>
+          <t>Populates `hr1_cur`, `hr1_month_label` in globals.</t>
+        </is>
+      </c>
+      <c r="E140" s="23" t="n"/>
+      <c r="F140" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G140" s="20" t="n"/>
+      <c r="H140" s="20" t="n"/>
+      <c r="I140" s="20" t="n"/>
+      <c r="J140" s="20" t="n"/>
+      <c r="K140" s="25" t="n"/>
+      <c r="L140" s="20" t="n"/>
+      <c r="M140" s="20" t="n"/>
+      <c r="N140" s="20" t="n"/>
+    </row>
+    <row r="141" ht="32" customHeight="1">
+      <c r="B141" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C141" s="21" t="inlineStr">
+        <is>
+          <t>sheets/inactivity_reasons.R — fetch_inactivity_reasons
+L23</t>
+        </is>
+      </c>
+      <c r="D141" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble with 7 reason codes.</t>
+        </is>
+      </c>
+      <c r="E141" s="23" t="n"/>
+      <c r="F141" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G141" s="20" t="n"/>
+      <c r="H141" s="20" t="n"/>
+      <c r="I141" s="20" t="n"/>
+      <c r="J141" s="20" t="n"/>
+      <c r="K141" s="25" t="n"/>
+      <c r="L141" s="20" t="n"/>
+      <c r="M141" s="20" t="n"/>
+      <c r="N141" s="20" t="n"/>
+    </row>
+    <row r="142" ht="32" customHeight="1">
+      <c r="B142" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C142" s="21" t="inlineStr">
+        <is>
+          <t>sheets/inactivity_reasons.R — compute_inactivity_reasons
+L37</t>
+        </is>
+      </c>
+      <c r="D142" s="22" t="inlineStr">
+        <is>
+          <t>Returns list with cur/dy/dc for each of the 7 reasons.</t>
+        </is>
+      </c>
+      <c r="E142" s="23" t="n"/>
+      <c r="F142" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G142" s="20" t="n"/>
+      <c r="H142" s="20" t="n"/>
+      <c r="I142" s="20" t="n"/>
+      <c r="J142" s="20" t="n"/>
+      <c r="K142" s="25" t="n"/>
+      <c r="L142" s="20" t="n"/>
+      <c r="M142" s="20" t="n"/>
+      <c r="N142" s="20" t="n"/>
+    </row>
+    <row r="143" ht="32" customHeight="1">
+      <c r="B143" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C143" s="21" t="inlineStr">
+        <is>
+          <t>sheets/inactivity_reasons.R — find_top_n_drivers
+L65</t>
+        </is>
+      </c>
+      <c r="D143" s="22" t="inlineStr">
+        <is>
+          <t>`find_top_n_drivers(df, 3)` returns top-3 reasons by absolute change magnitude.</t>
+        </is>
+      </c>
+      <c r="E143" s="23" t="n"/>
+      <c r="F143" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G143" s="20" t="n"/>
+      <c r="H143" s="20" t="n"/>
+      <c r="I143" s="20" t="n"/>
+      <c r="J143" s="20" t="n"/>
+      <c r="K143" s="25" t="n"/>
+      <c r="L143" s="20" t="n"/>
+      <c r="M143" s="20" t="n"/>
+      <c r="N143" s="20" t="n"/>
+    </row>
+    <row r="144" ht="32" customHeight="1">
+      <c r="B144" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C144" s="21" t="inlineStr">
+        <is>
+          <t>sheets/inactivity_reasons.R — generate_inactivity_driver_text
+L77</t>
+        </is>
+      </c>
+      <c r="D144" s="22" t="inlineStr">
+        <is>
+          <t>Returns natural-language string listing the top drivers (direction + magnitude).</t>
+        </is>
+      </c>
+      <c r="E144" s="23" t="n"/>
+      <c r="F144" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G144" s="20" t="n"/>
+      <c r="H144" s="20" t="n"/>
+      <c r="I144" s="20" t="n"/>
+      <c r="J144" s="20" t="n"/>
+      <c r="K144" s="25" t="n"/>
+      <c r="L144" s="20" t="n"/>
+      <c r="M144" s="20" t="n"/>
+      <c r="N144" s="20" t="n"/>
+    </row>
+    <row r="145" ht="32" customHeight="1">
+      <c r="B145" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C145" s="21" t="inlineStr">
+        <is>
+          <t>sheets/inactivity_reasons.R — calculate_inactivity_reasons
+L90</t>
+        </is>
+      </c>
+      <c r="D145" s="22" t="inlineStr">
+        <is>
+          <t>Populates inactivity globals consumed by summary.R.</t>
+        </is>
+      </c>
+      <c r="E145" s="23" t="n"/>
+      <c r="F145" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G145" s="20" t="n"/>
+      <c r="H145" s="20" t="n"/>
+      <c r="I145" s="20" t="n"/>
+      <c r="J145" s="20" t="n"/>
+      <c r="K145" s="25" t="n"/>
+      <c r="L145" s="20" t="n"/>
+      <c r="M145" s="20" t="n"/>
+      <c r="N145" s="20" t="n"/>
+    </row>
+    <row r="146" ht="32" customHeight="1">
+      <c r="B146" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C146" s="21" t="inlineStr">
+        <is>
+          <t>sheets/payroll_by_age.R — fetch_payroll_by_age
+L12</t>
+        </is>
+      </c>
+      <c r="D146" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble from ons.labour_market_employees_age.</t>
+        </is>
+      </c>
+      <c r="E146" s="23" t="n"/>
+      <c r="F146" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G146" s="20" t="n"/>
+      <c r="H146" s="20" t="n"/>
+      <c r="I146" s="20" t="n"/>
+      <c r="J146" s="20" t="n"/>
+      <c r="K146" s="25" t="n"/>
+      <c r="L146" s="20" t="n"/>
+      <c r="M146" s="20" t="n"/>
+      <c r="N146" s="20" t="n"/>
+    </row>
+    <row r="147" ht="32" customHeight="1">
+      <c r="B147" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C147" s="21" t="inlineStr">
+        <is>
+          <t>sheets/payroll_by_age.R — parse_month_label_to_date
+L26</t>
+        </is>
+      </c>
+      <c r="D147" s="22" t="inlineStr">
+        <is>
+          <t>Run `parse_month_label_to_date("january 2026")` → 2026-01-01.</t>
+        </is>
+      </c>
+      <c r="E147" s="23" t="n"/>
+      <c r="F147" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G147" s="20" t="n"/>
+      <c r="H147" s="20" t="n"/>
+      <c r="I147" s="20" t="n"/>
+      <c r="J147" s="20" t="n"/>
+      <c r="K147" s="25" t="n"/>
+      <c r="L147" s="20" t="n"/>
+      <c r="M147" s="20" t="n"/>
+      <c r="N147" s="20" t="n"/>
+    </row>
+    <row r="148" ht="32" customHeight="1">
+      <c r="B148" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C148" s="21" t="inlineStr">
+        <is>
+          <t>sheets/payroll_by_age.R — compute_payroll_by_age
+L31</t>
+        </is>
+      </c>
+      <c r="D148" s="22" t="inlineStr">
+        <is>
+          <t>Returns df with age group + level + change for latest period.</t>
+        </is>
+      </c>
+      <c r="E148" s="23" t="n"/>
+      <c r="F148" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G148" s="20" t="n"/>
+      <c r="H148" s="20" t="n"/>
+      <c r="I148" s="20" t="n"/>
+      <c r="J148" s="20" t="n"/>
+      <c r="K148" s="25" t="n"/>
+      <c r="L148" s="20" t="n"/>
+      <c r="M148" s="20" t="n"/>
+      <c r="N148" s="20" t="n"/>
+    </row>
+    <row r="149" ht="32" customHeight="1">
+      <c r="B149" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C149" s="21" t="inlineStr">
+        <is>
+          <t>sheets/payroll_by_age.R — calculate_payroll_by_age
+L52</t>
+        </is>
+      </c>
+      <c r="D149" s="22" t="inlineStr">
+        <is>
+          <t>Populates payroll-by-age globals.</t>
+        </is>
+      </c>
+      <c r="E149" s="23" t="n"/>
+      <c r="F149" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G149" s="20" t="n"/>
+      <c r="H149" s="20" t="n"/>
+      <c r="I149" s="20" t="n"/>
+      <c r="J149" s="20" t="n"/>
+      <c r="K149" s="25" t="n"/>
+      <c r="L149" s="20" t="n"/>
+      <c r="M149" s="20" t="n"/>
+      <c r="N149" s="20" t="n"/>
+    </row>
+    <row r="150" ht="32" customHeight="1">
+      <c r="B150" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C150" s="21" t="inlineStr">
+        <is>
+          <t>sheets/sector_payroll.R — fetch_sector_payroll
+L10</t>
+        </is>
+      </c>
+      <c r="D150" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble from ons.labour_market__employees_industry.</t>
+        </is>
+      </c>
+      <c r="E150" s="23" t="n"/>
+      <c r="F150" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G150" s="20" t="n"/>
+      <c r="H150" s="20" t="n"/>
+      <c r="I150" s="20" t="n"/>
+      <c r="J150" s="20" t="n"/>
+      <c r="K150" s="25" t="n"/>
+      <c r="L150" s="20" t="n"/>
+      <c r="M150" s="20" t="n"/>
+      <c r="N150" s="20" t="n"/>
+    </row>
+    <row r="151" ht="32" customHeight="1">
+      <c r="B151" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C151" s="21" t="inlineStr">
+        <is>
+          <t>sheets/sector_payroll.R — val_sector
+L24</t>
+        </is>
+      </c>
+      <c r="D151" s="22" t="inlineStr">
+        <is>
+          <t>Run `val_sector(df, "I", period)` (hospitality) returns numeric.</t>
+        </is>
+      </c>
+      <c r="E151" s="23" t="n"/>
+      <c r="F151" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G151" s="20" t="n"/>
+      <c r="H151" s="20" t="n"/>
+      <c r="I151" s="20" t="n"/>
+      <c r="J151" s="20" t="n"/>
+      <c r="K151" s="25" t="n"/>
+      <c r="L151" s="20" t="n"/>
+      <c r="M151" s="20" t="n"/>
+      <c r="N151" s="20" t="n"/>
+    </row>
+    <row r="152" ht="32" customHeight="1">
+      <c r="B152" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C152" s="21" t="inlineStr">
+        <is>
+          <t>sheets/sector_payroll.R — compute_sector
+L32</t>
+        </is>
+      </c>
+      <c r="D152" s="22" t="inlineStr">
+        <is>
+          <t>Returns cur + dy (YoY) for a single sector.</t>
+        </is>
+      </c>
+      <c r="E152" s="23" t="n"/>
+      <c r="F152" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G152" s="20" t="n"/>
+      <c r="H152" s="20" t="n"/>
+      <c r="I152" s="20" t="n"/>
+      <c r="J152" s="20" t="n"/>
+      <c r="K152" s="25" t="n"/>
+      <c r="L152" s="20" t="n"/>
+      <c r="M152" s="20" t="n"/>
+      <c r="N152" s="20" t="n"/>
+    </row>
+    <row r="153" ht="32" customHeight="1">
+      <c r="B153" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C153" s="21" t="inlineStr">
+        <is>
+          <t>sheets/sector_payroll.R — calculate_sector_payroll
+L57</t>
+        </is>
+      </c>
+      <c r="D153" s="22" t="inlineStr">
+        <is>
+          <t>Populates `hosp_dy`, `retail_dy`, `health_dy` (SIC I, G, Q).</t>
+        </is>
+      </c>
+      <c r="E153" s="23" t="n"/>
+      <c r="F153" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G153" s="20" t="n"/>
+      <c r="H153" s="20" t="n"/>
+      <c r="I153" s="20" t="n"/>
+      <c r="J153" s="20" t="n"/>
+      <c r="K153" s="25" t="n"/>
+      <c r="L153" s="20" t="n"/>
+      <c r="M153" s="20" t="n"/>
+      <c r="N153" s="20" t="n"/>
+    </row>
+    <row r="154" ht="32" customHeight="1">
+      <c r="B154" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C154" s="21" t="inlineStr">
+        <is>
+          <t>sheets/unemployment_by_age.R — fetch_unemployment_by_age
+L11</t>
+        </is>
+      </c>
+      <c r="D154" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble from ons.labour_market_unemployment.</t>
+        </is>
+      </c>
+      <c r="E154" s="23" t="n"/>
+      <c r="F154" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G154" s="20" t="n"/>
+      <c r="H154" s="20" t="n"/>
+      <c r="I154" s="20" t="n"/>
+      <c r="J154" s="20" t="n"/>
+      <c r="K154" s="25" t="n"/>
+      <c r="L154" s="20" t="n"/>
+      <c r="M154" s="20" t="n"/>
+      <c r="N154" s="20" t="n"/>
+    </row>
+    <row r="155" ht="32" customHeight="1">
+      <c r="B155" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C155" s="21" t="inlineStr">
+        <is>
+          <t>sheets/unemployment_by_age.R — parse_lfs_period_to_end_date
+L29</t>
+        </is>
+      </c>
+      <c r="D155" s="22" t="inlineStr">
+        <is>
+          <t>Run `parse_lfs_period_to_end_date("mar-may 1992")` → 1992-05-01.</t>
+        </is>
+      </c>
+      <c r="E155" s="23" t="n"/>
+      <c r="F155" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G155" s="20" t="n"/>
+      <c r="H155" s="20" t="n"/>
+      <c r="I155" s="20" t="n"/>
+      <c r="J155" s="20" t="n"/>
+      <c r="K155" s="25" t="n"/>
+      <c r="L155" s="20" t="n"/>
+      <c r="M155" s="20" t="n"/>
+      <c r="N155" s="20" t="n"/>
+    </row>
+    <row r="156" ht="32" customHeight="1">
+      <c r="B156" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C156" s="21" t="inlineStr">
+        <is>
+          <t>sheets/unemployment_by_age.R — compute_unemployment_by_age
+L41</t>
+        </is>
+      </c>
+      <c r="D156" s="22" t="inlineStr">
+        <is>
+          <t>Returns df with age groups + values for latest period.</t>
+        </is>
+      </c>
+      <c r="E156" s="23" t="n"/>
+      <c r="F156" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G156" s="20" t="n"/>
+      <c r="H156" s="20" t="n"/>
+      <c r="I156" s="20" t="n"/>
+      <c r="J156" s="20" t="n"/>
+      <c r="K156" s="25" t="n"/>
+      <c r="L156" s="20" t="n"/>
+      <c r="M156" s="20" t="n"/>
+      <c r="N156" s="20" t="n"/>
+    </row>
+    <row r="157" ht="32" customHeight="1">
+      <c r="B157" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C157" s="21" t="inlineStr">
+        <is>
+          <t>sheets/unemployment_by_age.R — calculate_unemployment_by_age
+L69</t>
+        </is>
+      </c>
+      <c r="D157" s="22" t="inlineStr">
+        <is>
+          <t>Populates unemployment-by-age globals.</t>
+        </is>
+      </c>
+      <c r="E157" s="23" t="n"/>
+      <c r="F157" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G157" s="20" t="n"/>
+      <c r="H157" s="20" t="n"/>
+      <c r="I157" s="20" t="n"/>
+      <c r="J157" s="20" t="n"/>
+      <c r="K157" s="25" t="n"/>
+      <c r="L157" s="20" t="n"/>
+      <c r="M157" s="20" t="n"/>
+      <c r="N157" s="20" t="n"/>
+    </row>
+    <row r="158" ht="32" customHeight="1">
+      <c r="B158" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C158" s="21" t="inlineStr">
+        <is>
+          <t>sheets/workforce_jobs.R — fetch_workforce_jobs
+L12</t>
+        </is>
+      </c>
+      <c r="D158" s="22" t="inlineStr">
+        <is>
+          <t>Returns tibble from ons.labour_market_workforce_jobs.</t>
+        </is>
+      </c>
+      <c r="E158" s="23" t="n"/>
+      <c r="F158" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G158" s="20" t="n"/>
+      <c r="H158" s="20" t="n"/>
+      <c r="I158" s="20" t="n"/>
+      <c r="J158" s="20" t="n"/>
+      <c r="K158" s="25" t="n"/>
+      <c r="L158" s="20" t="n"/>
+      <c r="M158" s="20" t="n"/>
+      <c r="N158" s="20" t="n"/>
+    </row>
+    <row r="159" ht="32" customHeight="1">
+      <c r="B159" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C159" s="21" t="inlineStr">
+        <is>
+          <t>sheets/workforce_jobs.R — parse_wfj_period_to_date
+L27</t>
+        </is>
+      </c>
+      <c r="D159" s="22" t="inlineStr">
+        <is>
+          <t>Run `parse_wfj_period_to_date("mar 98 (r)")` → 1998-03-01; `"mar 25"` → 2025-03-01.</t>
+        </is>
+      </c>
+      <c r="E159" s="23" t="n"/>
+      <c r="F159" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G159" s="20" t="n"/>
+      <c r="H159" s="20" t="n"/>
+      <c r="I159" s="20" t="n"/>
+      <c r="J159" s="20" t="n"/>
+      <c r="K159" s="25" t="n"/>
+      <c r="L159" s="20" t="n"/>
+      <c r="M159" s="20" t="n"/>
+      <c r="N159" s="20" t="n"/>
+    </row>
+    <row r="160" ht="32" customHeight="1">
+      <c r="B160" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C160" s="21" t="inlineStr">
+        <is>
+          <t>sheets/workforce_jobs.R — latest_wfj_period_label
+L40</t>
+        </is>
+      </c>
+      <c r="D160" s="22" t="inlineStr">
+        <is>
+          <t>Returns most recent period label string.</t>
+        </is>
+      </c>
+      <c r="E160" s="23" t="n"/>
+      <c r="F160" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G160" s="20" t="n"/>
+      <c r="H160" s="20" t="n"/>
+      <c r="I160" s="20" t="n"/>
+      <c r="J160" s="20" t="n"/>
+      <c r="K160" s="25" t="n"/>
+      <c r="L160" s="20" t="n"/>
+      <c r="M160" s="20" t="n"/>
+      <c r="N160" s="20" t="n"/>
+    </row>
+    <row r="161" ht="32" customHeight="1">
+      <c r="B161" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C161" s="21" t="inlineStr">
+        <is>
+          <t>sheets/workforce_jobs.R — compute_workforce_jobs
+L50</t>
+        </is>
+      </c>
+      <c r="D161" s="22" t="inlineStr">
+        <is>
+          <t>Returns totals + by-industry df for latest period.</t>
+        </is>
+      </c>
+      <c r="E161" s="23" t="n"/>
+      <c r="F161" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G161" s="20" t="n"/>
+      <c r="H161" s="20" t="n"/>
+      <c r="I161" s="20" t="n"/>
+      <c r="J161" s="20" t="n"/>
+      <c r="K161" s="25" t="n"/>
+      <c r="L161" s="20" t="n"/>
+      <c r="M161" s="20" t="n"/>
+      <c r="N161" s="20" t="n"/>
+    </row>
+    <row r="162" ht="32" customHeight="1">
+      <c r="B162" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C162" s="21" t="inlineStr">
+        <is>
+          <t>sheets/workforce_jobs.R — calculate_workforce_jobs
+L77</t>
+        </is>
+      </c>
+      <c r="D162" s="22" t="inlineStr">
+        <is>
+          <t>Populates workforce-jobs globals.</t>
+        </is>
+      </c>
+      <c r="E162" s="23" t="n"/>
+      <c r="F162" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G162" s="20" t="n"/>
+      <c r="H162" s="20" t="n"/>
+      <c r="I162" s="20" t="n"/>
+      <c r="J162" s="20" t="n"/>
+      <c r="K162" s="25" t="n"/>
+      <c r="L162" s="20" t="n"/>
+      <c r="M162" s="20" t="n"/>
+      <c r="N162" s="20" t="n"/>
+    </row>
+    <row r="163" ht="32" customHeight="1">
+      <c r="B163" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C163" s="21" t="inlineStr">
+        <is>
+          <t>sheets/summary.R — calc_workforce_jobs_changes
+L12</t>
+        </is>
+      </c>
+      <c r="D163" s="22" t="inlineStr">
+        <is>
+          <t>Returns cur/dq/dy/pct_q/pct_y for total WFJ.</t>
+        </is>
+      </c>
+      <c r="E163" s="23" t="n"/>
+      <c r="F163" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G163" s="20" t="n"/>
+      <c r="H163" s="20" t="n"/>
+      <c r="I163" s="20" t="n"/>
+      <c r="J163" s="20" t="n"/>
+      <c r="K163" s="25" t="n"/>
+      <c r="L163" s="20" t="n"/>
+      <c r="M163" s="20" t="n"/>
+      <c r="N163" s="20" t="n"/>
+    </row>
+    <row r="164" ht="32" customHeight="1">
+      <c r="B164" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C164" s="21" t="inlineStr">
+        <is>
+          <t>sheets/summary.R — calc_youth_unemp
+L59</t>
+        </is>
+      </c>
+      <c r="D164" s="22" t="inlineStr">
+        <is>
+          <t>Returns level/dq/largest_since_2022 flag for 18-24 unemployment.</t>
+        </is>
+      </c>
+      <c r="E164" s="23" t="n"/>
+      <c r="F164" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G164" s="20" t="n"/>
+      <c r="H164" s="20" t="n"/>
+      <c r="I164" s="20" t="n"/>
+      <c r="J164" s="20" t="n"/>
+      <c r="K164" s="25" t="n"/>
+      <c r="L164" s="20" t="n"/>
+      <c r="M164" s="20" t="n"/>
+      <c r="N164" s="20" t="n"/>
+    </row>
+    <row r="165" ht="32" customHeight="1">
+      <c r="B165" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C165" s="21" t="inlineStr">
+        <is>
+          <t>sheets/summary.R — calc_payroll_age_drops
+L110</t>
+        </is>
+      </c>
+      <c r="D165" s="22" t="inlineStr">
+        <is>
+          <t>Returns top-3 age groups by largest monthly payroll drop.</t>
+        </is>
+      </c>
+      <c r="E165" s="23" t="n"/>
+      <c r="F165" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G165" s="20" t="n"/>
+      <c r="H165" s="20" t="n"/>
+      <c r="I165" s="20" t="n"/>
+      <c r="J165" s="20" t="n"/>
+      <c r="K165" s="25" t="n"/>
+      <c r="L165" s="20" t="n"/>
+      <c r="M165" s="20" t="n"/>
+      <c r="N165" s="20" t="n"/>
+    </row>
+    <row r="166" ht="32" customHeight="1">
+      <c r="B166" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C166" s="21" t="inlineStr">
+        <is>
+          <t>sheets/summary.R — generate_summary
+L157</t>
+        </is>
+      </c>
+      <c r="D166" s="22" t="inlineStr">
+        <is>
+          <t>Returns list of 10 narrative line strings.</t>
+        </is>
+      </c>
+      <c r="E166" s="23" t="n"/>
+      <c r="F166" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G166" s="20" t="n"/>
+      <c r="H166" s="20" t="n"/>
+      <c r="I166" s="20" t="n"/>
+      <c r="J166" s="20" t="n"/>
+      <c r="K166" s="25" t="n"/>
+      <c r="L166" s="20" t="n"/>
+      <c r="M166" s="20" t="n"/>
+      <c r="N166" s="20" t="n"/>
+    </row>
+    <row r="167" ht="32" customHeight="1">
+      <c r="B167" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C167" s="21" t="inlineStr">
+        <is>
+          <t>sheets/top_ten_stats.R — dir_word
+L7</t>
+        </is>
+      </c>
+      <c r="D167" s="22" t="inlineStr">
+        <is>
+          <t>Run `dir_word(1)` → "an increase of"; `dir_word(-1)` → "a decrease of"; `dir_word(0)` → "no change,".</t>
+        </is>
+      </c>
+      <c r="E167" s="23" t="n"/>
+      <c r="F167" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G167" s="20" t="n"/>
+      <c r="H167" s="20" t="n"/>
+      <c r="I167" s="20" t="n"/>
+      <c r="J167" s="20" t="n"/>
+      <c r="K167" s="25" t="n"/>
+      <c r="L167" s="20" t="n"/>
+      <c r="M167" s="20" t="n"/>
+      <c r="N167" s="20" t="n"/>
+    </row>
+    <row r="168" ht="32" customHeight="1">
+      <c r="B168" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C168" s="21" t="inlineStr">
+        <is>
+          <t>sheets/top_ten_stats.R — fmt_int_1k_top10
+L15</t>
+        </is>
+      </c>
+      <c r="D168" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_int_1k_top10(123456)` → "123,000" (rounded to nearest 1k).</t>
+        </is>
+      </c>
+      <c r="E168" s="23" t="n"/>
+      <c r="F168" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G168" s="20" t="n"/>
+      <c r="H168" s="20" t="n"/>
+      <c r="I168" s="20" t="n"/>
+      <c r="J168" s="20" t="n"/>
+      <c r="K168" s="25" t="n"/>
+      <c r="L168" s="20" t="n"/>
+      <c r="M168" s="20" t="n"/>
+      <c r="N168" s="20" t="n"/>
+    </row>
+    <row r="169" ht="32" customHeight="1">
+      <c r="B169" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C169" s="21" t="inlineStr">
+        <is>
+          <t>sheets/top_ten_stats.R — fmt_flash_change
+L21</t>
+        </is>
+      </c>
+      <c r="D169" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_flash_change(1.5)` → "2,000" (1500 rounded to nearest 1k).</t>
+        </is>
+      </c>
+      <c r="E169" s="23" t="n"/>
+      <c r="F169" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G169" s="20" t="n"/>
+      <c r="H169" s="20" t="n"/>
+      <c r="I169" s="20" t="n"/>
+      <c r="J169" s="20" t="n"/>
+      <c r="K169" s="25" t="n"/>
+      <c r="L169" s="20" t="n"/>
+      <c r="M169" s="20" t="n"/>
+      <c r="N169" s="20" t="n"/>
+    </row>
+    <row r="170" ht="32" customHeight="1">
+      <c r="B170" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C170" s="21" t="inlineStr">
+        <is>
+          <t>sheets/top_ten_stats.R — fmt_rate
+L26</t>
+        </is>
+      </c>
+      <c r="D170" s="22" t="inlineStr">
+        <is>
+          <t>Run `fmt_rate(74.95)` → "75.0" (1dp).</t>
+        </is>
+      </c>
+      <c r="E170" s="23" t="n"/>
+      <c r="F170" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G170" s="20" t="n"/>
+      <c r="H170" s="20" t="n"/>
+      <c r="I170" s="20" t="n"/>
+      <c r="J170" s="20" t="n"/>
+      <c r="K170" s="25" t="n"/>
+      <c r="L170" s="20" t="n"/>
+      <c r="M170" s="20" t="n"/>
+      <c r="N170" s="20" t="n"/>
+    </row>
+    <row r="171" ht="32" customHeight="1">
+      <c r="B171" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C171" s="21" t="inlineStr">
+        <is>
+          <t>sheets/top_ten_stats.R — generate_top_ten
+L31</t>
+        </is>
+      </c>
+      <c r="D171" s="22" t="inlineStr">
+        <is>
+          <t>Returns list(line1..line10) with narrative strings; catches errors and returns fallback text.</t>
+        </is>
+      </c>
+      <c r="E171" s="23" t="n"/>
+      <c r="F171" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G171" s="20" t="n"/>
+      <c r="H171" s="20" t="n"/>
+      <c r="I171" s="20" t="n"/>
+      <c r="J171" s="20" t="n"/>
+      <c r="K171" s="25" t="n"/>
+      <c r="L171" s="20" t="n"/>
+      <c r="M171" s="20" t="n"/>
+      <c r="N171" s="20" t="n"/>
+    </row>
+    <row r="172" ht="32" customHeight="1">
+      <c r="B172" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C172" s="21" t="inlineStr">
+        <is>
+          <t>sheets/excel_audit_workbook.R — .safe_read
+L12</t>
+        </is>
+      </c>
+      <c r="D172" s="22" t="inlineStr">
+        <is>
+          <t>Reads sheet preserving ONS suppression markers ("..", "[c]", etc.) as text, not NA.</t>
+        </is>
+      </c>
+      <c r="E172" s="23" t="n"/>
+      <c r="F172" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G172" s="20" t="n"/>
+      <c r="H172" s="20" t="n"/>
+      <c r="I172" s="20" t="n"/>
+      <c r="J172" s="20" t="n"/>
+      <c r="K172" s="25" t="n"/>
+      <c r="L172" s="20" t="n"/>
+      <c r="M172" s="20" t="n"/>
+      <c r="N172" s="20" t="n"/>
+    </row>
+    <row r="173" ht="32" customHeight="1">
+      <c r="B173" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C173" s="21" t="inlineStr">
+        <is>
+          <t>sheets/excel_audit_workbook.R — .first_num_r
+L48</t>
+        </is>
+      </c>
+      <c r="D173" s="22" t="inlineStr">
+        <is>
+          <t>Returns row index of first numeric value in column.</t>
+        </is>
+      </c>
+      <c r="E173" s="23" t="n"/>
+      <c r="F173" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G173" s="20" t="n"/>
+      <c r="H173" s="20" t="n"/>
+      <c r="I173" s="20" t="n"/>
+      <c r="J173" s="20" t="n"/>
+      <c r="K173" s="25" t="n"/>
+      <c r="L173" s="20" t="n"/>
+      <c r="M173" s="20" t="n"/>
+      <c r="N173" s="20" t="n"/>
+    </row>
+    <row r="174" ht="32" customHeight="1">
+      <c r="B174" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C174" s="21" t="inlineStr">
+        <is>
+          <t>sheets/excel_audit_workbook.R — .lfs_metric
+L54</t>
+        </is>
+      </c>
+      <c r="D174" s="22" t="inlineStr">
+        <is>
+          <t>Extracts cur/q/y/covid/elec values from column and computes dq/dy/dc/de deltas (the "Labometric" JB asked about).</t>
+        </is>
+      </c>
+      <c r="E174" s="23" t="n"/>
+      <c r="F174" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G174" s="20" t="n"/>
+      <c r="H174" s="20" t="n"/>
+      <c r="I174" s="20" t="n"/>
+      <c r="J174" s="20" t="n"/>
+      <c r="K174" s="25" t="n"/>
+      <c r="L174" s="20" t="n"/>
+      <c r="M174" s="20" t="n"/>
+      <c r="N174" s="20" t="n"/>
+    </row>
+    <row r="175" ht="32" customHeight="1">
+      <c r="B175" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C175" s="21" t="inlineStr">
+        <is>
+          <t>sheets/excel_audit_workbook.R — .restore_text
+L63</t>
+        </is>
+      </c>
+      <c r="D175" s="22" t="inlineStr">
+        <is>
+          <t>Re-inserts suppression markers that got coerced to NA during numeric conversion.</t>
+        </is>
+      </c>
+      <c r="E175" s="23" t="n"/>
+      <c r="F175" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G175" s="20" t="n"/>
+      <c r="H175" s="20" t="n"/>
+      <c r="I175" s="20" t="n"/>
+      <c r="J175" s="20" t="n"/>
+      <c r="K175" s="25" t="n"/>
+      <c r="L175" s="20" t="n"/>
+      <c r="M175" s="20" t="n"/>
+      <c r="N175" s="20" t="n"/>
+    </row>
+    <row r="176" ht="32" customHeight="1">
+      <c r="B176" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C176" s="21" t="inlineStr">
+        <is>
+          <t>sheets/excel_audit_workbook.R — .trim_source
+L78</t>
+        </is>
+      </c>
+      <c r="D176" s="22" t="inlineStr">
+        <is>
+          <t>Strips header/footnote rows; returns df with data rows only.</t>
+        </is>
+      </c>
+      <c r="E176" s="23" t="n"/>
+      <c r="F176" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G176" s="20" t="n"/>
+      <c r="H176" s="20" t="n"/>
+      <c r="I176" s="20" t="n"/>
+      <c r="J176" s="20" t="n"/>
+      <c r="K176" s="25" t="n"/>
+      <c r="L176" s="20" t="n"/>
+      <c r="M176" s="20" t="n"/>
+      <c r="N176" s="20" t="n"/>
+    </row>
+    <row r="177" ht="32" customHeight="1">
+      <c r="B177" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C177" s="21" t="inlineStr">
+        <is>
+          <t>sheets/excel_audit_workbook.R — .col_letter
+L113</t>
+        </is>
+      </c>
+      <c r="D177" s="22" t="inlineStr">
+        <is>
+          <t>Run `.col_letter(1)` → "A"; `.col_letter(28)` → "AB"; `.col_letter(702)` → "ZZ".</t>
+        </is>
+      </c>
+      <c r="E177" s="23" t="n"/>
+      <c r="F177" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G177" s="20" t="n"/>
+      <c r="H177" s="20" t="n"/>
+      <c r="I177" s="20" t="n"/>
+      <c r="J177" s="20" t="n"/>
+      <c r="K177" s="25" t="n"/>
+      <c r="L177" s="20" t="n"/>
+      <c r="M177" s="20" t="n"/>
+      <c r="N177" s="20" t="n"/>
+    </row>
+    <row r="178" ht="32" customHeight="1">
+      <c r="B178" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C178" s="21" t="inlineStr">
+        <is>
+          <t>sheets/excel_audit_workbook.R — .find_output_row
+L123</t>
+        </is>
+      </c>
+      <c r="D178" s="22" t="inlineStr">
+        <is>
+          <t>Given label + df, returns matching row index or NA.</t>
+        </is>
+      </c>
+      <c r="E178" s="23" t="n"/>
+      <c r="F178" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G178" s="20" t="n"/>
+      <c r="H178" s="20" t="n"/>
+      <c r="I178" s="20" t="n"/>
+      <c r="J178" s="20" t="n"/>
+      <c r="K178" s="25" t="n"/>
+      <c r="L178" s="20" t="n"/>
+      <c r="M178" s="20" t="n"/>
+      <c r="N178" s="20" t="n"/>
+    </row>
+    <row r="179" ht="32" customHeight="1">
+      <c r="B179" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C179" s="21" t="inlineStr">
+        <is>
+          <t>sheets/excel_audit_workbook.R — .find_output_row_date
+L130</t>
+        </is>
+      </c>
+      <c r="D179" s="22" t="inlineStr">
+        <is>
+          <t>Matches date column to target date; returns row index or NA.</t>
+        </is>
+      </c>
+      <c r="E179" s="23" t="n"/>
+      <c r="F179" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G179" s="20" t="n"/>
+      <c r="H179" s="20" t="n"/>
+      <c r="I179" s="20" t="n"/>
+      <c r="J179" s="20" t="n"/>
+      <c r="K179" s="25" t="n"/>
+      <c r="L179" s="20" t="n"/>
+      <c r="M179" s="20" t="n"/>
+      <c r="N179" s="20" t="n"/>
+    </row>
+    <row r="180" ht="32" customHeight="1">
+      <c r="B180" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C180" s="21" t="inlineStr">
+        <is>
+          <t>sheets/excel_audit_workbook.R — .detect_sheet
+L278</t>
+        </is>
+      </c>
+      <c r="D180" s="22" t="inlineStr">
+        <is>
+          <t>Returns first matching sheet name from candidates list; NULL if none match.</t>
+        </is>
+      </c>
+      <c r="E180" s="23" t="n"/>
+      <c r="F180" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G180" s="20" t="n"/>
+      <c r="H180" s="20" t="n"/>
+      <c r="I180" s="20" t="n"/>
+      <c r="J180" s="20" t="n"/>
+      <c r="K180" s="25" t="n"/>
+      <c r="L180" s="20" t="n"/>
+      <c r="M180" s="20" t="n"/>
+      <c r="N180" s="20" t="n"/>
+    </row>
+    <row r="181" ht="32" customHeight="1">
+      <c r="B181" s="20" t="inlineStr">
+        <is>
+          <t>v0.2</t>
+        </is>
+      </c>
+      <c r="C181" s="21" t="inlineStr">
+        <is>
+          <t>sheets/excel_audit_workbook.R — create_audit_workbook
+L301</t>
+        </is>
+      </c>
+      <c r="D181" s="22" t="inlineStr">
+        <is>
+          <t>Produces audit .xlsx workbook with all formulas calculated and suppression markers preserved.</t>
+        </is>
+      </c>
+      <c r="E181" s="23" t="n"/>
+      <c r="F181" s="24" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="G181" s="20" t="n"/>
+      <c r="H181" s="20" t="n"/>
+      <c r="I181" s="20" t="n"/>
+      <c r="J181" s="20" t="n"/>
+      <c r="K181" s="25" t="n"/>
+      <c r="L181" s="20" t="n"/>
+      <c r="M181" s="20" t="n"/>
+      <c r="N181" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>